<commit_message>
supprime doubllon de excel ville et modification du version de chrome
</commit_message>
<xml_diff>
--- a/src/citys/us_cities_sample.xlsx
+++ b/src/citys/us_cities_sample.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\DNS\src\citys\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CED49A-2705-4887-9295-CB79AF419EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B55158-5043-4D55-8DFF-4EBB93C83F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="US Cities" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="345">
   <si>
     <t>8,478,072</t>
   </si>
@@ -20451,15 +20451,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>9525</xdr:colOff>
       <xdr:row>333</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>165100</xdr:colOff>
-      <xdr:row>333</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>174625</xdr:colOff>
+      <xdr:row>334</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -20489,7 +20489,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5486400" y="150348950"/>
+          <a:off x="1819275" y="63493650"/>
           <a:ext cx="165100" cy="165100"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -21590,14 +21590,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B347"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B333"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>311</v>
       </c>
@@ -21605,7 +21605,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>313</v>
       </c>
@@ -21613,7 +21613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -21621,7 +21621,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -21629,7 +21629,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -21637,7 +21637,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -21645,7 +21645,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>315</v>
       </c>
@@ -21653,7 +21653,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -21661,7 +21661,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -21669,7 +21669,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -21677,7 +21677,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>314</v>
       </c>
@@ -21685,7 +21685,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -21693,7 +21693,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -21701,7 +21701,7 @@
         <v>997.36800000000005</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -21709,7 +21709,7 @@
         <v>993.58799999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -21717,7 +21717,7 @@
         <v>943.476</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -21725,7 +21725,7 @@
         <v>933.26300000000003</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>316</v>
       </c>
@@ -21733,7 +21733,7 @@
         <v>891.48400000000004</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>317</v>
       </c>
@@ -21741,7 +21741,7 @@
         <v>827.52599999999995</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -21749,7 +21749,7 @@
         <v>780.995</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>318</v>
       </c>
@@ -21757,7 +21757,7 @@
         <v>729.01900000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -21765,7 +21765,7 @@
         <v>712.91899999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>319</v>
       </c>
@@ -21773,7 +21773,7 @@
         <v>704.96299999999997</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>320</v>
       </c>
@@ -21781,7 +21781,7 @@
         <v>702.25</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -21789,7 +21789,7 @@
         <v>681.72299999999996</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -21797,7 +21797,7 @@
         <v>678.92200000000003</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -21805,7 +21805,7 @@
         <v>673.45799999999997</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -21813,7 +21813,7 @@
         <v>645.70500000000004</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>321</v>
       </c>
@@ -21821,7 +21821,7 @@
         <v>640.79600000000005</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -21829,7 +21829,7 @@
         <v>635.74900000000002</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -21837,7 +21837,7 @@
         <v>610.91899999999998</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>322</v>
       </c>
@@ -21845,7 +21845,7 @@
         <v>568.27099999999996</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -21853,7 +21853,7 @@
         <v>563.53099999999995</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -21861,7 +21861,7 @@
         <v>560.32600000000002</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -21869,7 +21869,7 @@
         <v>554.01300000000003</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -21877,7 +21877,7 @@
         <v>550.10500000000002</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -21885,7 +21885,7 @@
         <v>535.798</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -21893,7 +21893,7 @@
         <v>520.07000000000005</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -21901,7 +21901,7 @@
         <v>517.15099999999995</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -21909,7 +21909,7 @@
         <v>516.03200000000004</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -21917,7 +21917,7 @@
         <v>499.82499999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -21925,7 +21925,7 @@
         <v>493.55399999999997</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -21933,7 +21933,7 @@
         <v>489.26499999999999</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -21941,7 +21941,7 @@
         <v>487.01400000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>323</v>
       </c>
@@ -21949,7 +21949,7 @@
         <v>454.80799999999999</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>43</v>
       </c>
@@ -21957,7 +21957,7 @@
         <v>450.90100000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>44</v>
       </c>
@@ -21965,7 +21965,7 @@
         <v>443.55399999999997</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>45</v>
       </c>
@@ -21973,7 +21973,7 @@
         <v>428.57900000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>46</v>
       </c>
@@ -21981,7 +21981,7 @@
         <v>417.46800000000002</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>47</v>
       </c>
@@ -21989,7 +21989,7 @@
         <v>415.154</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>48</v>
       </c>
@@ -21997,7 +21997,7 @@
         <v>414.54700000000003</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>49</v>
       </c>
@@ -22005,7 +22005,7 @@
         <v>403.67200000000003</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>50</v>
       </c>
@@ -22013,7 +22013,7 @@
         <v>403.13</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>51</v>
       </c>
@@ -22021,7 +22021,7 @@
         <v>400.99099999999999</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>52</v>
       </c>
@@ -22029,7 +22029,7 @@
         <v>365.37900000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>324</v>
       </c>
@@ -22037,7 +22037,7 @@
         <v>362.70100000000002</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>53</v>
       </c>
@@ -22045,7 +22045,7 @@
         <v>350.03899999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>325</v>
       </c>
@@ -22053,7 +22053,7 @@
         <v>344.96699999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>54</v>
       </c>
@@ -22061,7 +22061,7 @@
         <v>344.56099999999998</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>55</v>
       </c>
@@ -22069,7 +22069,7 @@
         <v>334.85399999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>326</v>
       </c>
@@ -22077,7 +22077,7 @@
         <v>329.43700000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>56</v>
       </c>
@@ -22085,7 +22085,7 @@
         <v>324.97500000000002</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>57</v>
       </c>
@@ -22093,7 +22093,7 @@
         <v>323.75700000000001</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>58</v>
       </c>
@@ -22101,7 +22101,7 @@
         <v>318.68299999999999</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>59</v>
       </c>
@@ -22109,7 +22109,7 @@
         <v>317.31700000000001</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>60</v>
       </c>
@@ -22117,7 +22117,7 @@
         <v>317.303</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>61</v>
       </c>
@@ -22125,7 +22125,7 @@
         <v>316.18400000000003</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>62</v>
       </c>
@@ -22133,7 +22133,7 @@
         <v>314.91500000000002</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>63</v>
       </c>
@@ -22141,7 +22141,7 @@
         <v>307.66800000000001</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>64</v>
       </c>
@@ -22149,7 +22149,7 @@
         <v>307.46499999999997</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>65</v>
       </c>
@@ -22157,7 +22157,7 @@
         <v>307.38099999999997</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>66</v>
       </c>
@@ -22165,7 +22165,7 @@
         <v>302.82400000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>67</v>
       </c>
@@ -22173,7 +22173,7 @@
         <v>301.87</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>68</v>
       </c>
@@ -22181,7 +22181,7 @@
         <v>300.61900000000003</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>69</v>
       </c>
@@ -22189,7 +22189,7 @@
         <v>294.03399999999999</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>70</v>
       </c>
@@ -22197,7 +22197,7 @@
         <v>293.286</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>342</v>
       </c>
@@ -22205,7 +22205,7 @@
         <v>289.60000000000002</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>71</v>
       </c>
@@ -22213,7 +22213,7 @@
         <v>288.79000000000002</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>72</v>
       </c>
@@ -22221,7 +22221,7 @@
         <v>285.3</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>73</v>
       </c>
@@ -22229,7 +22229,7 @@
         <v>281.714</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>74</v>
       </c>
@@ -22237,7 +22237,7 @@
         <v>281.23099999999999</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>327</v>
       </c>
@@ -22245,7 +22245,7 @@
         <v>279.69499999999999</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>75</v>
       </c>
@@ -22253,7 +22253,7 @@
         <v>278.54599999999999</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>76</v>
       </c>
@@ -22261,7 +22261,7 @@
         <v>276.61700000000002</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>77</v>
       </c>
@@ -22269,7 +22269,7 @@
         <v>273.20299999999997</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>78</v>
       </c>
@@ -22277,7 +22277,7 @@
         <v>272.08600000000001</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>79</v>
       </c>
@@ -22285,7 +22285,7 @@
         <v>267.10199999999998</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>80</v>
       </c>
@@ -22293,7 +22293,7 @@
         <v>265.63799999999998</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>81</v>
       </c>
@@ -22301,7 +22301,7 @@
         <v>261.26</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>82</v>
       </c>
@@ -22309,7 +22309,7 @@
         <v>258.57499999999999</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>83</v>
       </c>
@@ -22317,7 +22317,7 @@
         <v>258.14299999999997</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>84</v>
       </c>
@@ -22325,7 +22325,7 @@
         <v>258.06</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>85</v>
       </c>
@@ -22333,7 +22333,7 @@
         <v>255.76900000000001</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>329</v>
       </c>
@@ -22341,7 +22341,7 @@
         <v>254.99700000000001</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>86</v>
       </c>
@@ -22349,7 +22349,7 @@
         <v>250.43100000000001</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>87</v>
       </c>
@@ -22357,7 +22357,7 @@
         <v>246.17</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>328</v>
       </c>
@@ -22365,7 +22365,7 @@
         <v>237.96299999999999</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>88</v>
       </c>
@@ -22373,7 +22373,7 @@
         <v>235.38800000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>89</v>
       </c>
@@ -22381,7 +22381,7 @@
         <v>235.208</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>242</v>
       </c>
@@ -22389,7 +22389,7 @@
         <v>233.655</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>90</v>
       </c>
@@ -22397,7 +22397,7 @@
         <v>233.02500000000001</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>330</v>
       </c>
@@ -22405,7 +22405,7 @@
         <v>231.10499999999999</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>91</v>
       </c>
@@ -22413,7 +22413,7 @@
         <v>230.60900000000001</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>92</v>
       </c>
@@ -22421,7 +22421,7 @@
         <v>230.40199999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>93</v>
       </c>
@@ -22429,7 +22429,7 @@
         <v>229.15899999999999</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>94</v>
       </c>
@@ -22437,7 +22437,7 @@
         <v>228.202</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>95</v>
       </c>
@@ -22445,7 +22445,7 @@
         <v>228.19200000000001</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>96</v>
       </c>
@@ -22453,7 +22453,7 @@
         <v>227.52600000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>97</v>
       </c>
@@ -22461,7 +22461,7 @@
         <v>224.77500000000001</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>331</v>
       </c>
@@ -22469,7 +22469,7 @@
         <v>220.90700000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>98</v>
       </c>
@@ -22477,7 +22477,7 @@
         <v>220.59200000000001</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>99</v>
       </c>
@@ -22485,7 +22485,7 @@
         <v>218.45500000000001</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>100</v>
       </c>
@@ -22493,7 +22493,7 @@
         <v>217.78299999999999</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>101</v>
       </c>
@@ -22501,7 +22501,7 @@
         <v>213.91900000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>102</v>
       </c>
@@ -22509,7 +22509,7 @@
         <v>213.096</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>103</v>
       </c>
@@ -22517,7 +22517,7 @@
         <v>211.286</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>104</v>
       </c>
@@ -22525,7 +22525,7 @@
         <v>211.04</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>105</v>
       </c>
@@ -22533,7 +22533,7 @@
         <v>209.49600000000001</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>106</v>
       </c>
@@ -22541,7 +22541,7 @@
         <v>209.28899999999999</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>107</v>
       </c>
@@ -22549,7 +22549,7 @@
         <v>207.33099999999999</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>108</v>
       </c>
@@ -22557,7 +22557,7 @@
         <v>207.28200000000001</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>109</v>
       </c>
@@ -22565,7 +22565,7 @@
         <v>205.089</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>110</v>
       </c>
@@ -22573,7 +22573,7 @@
         <v>204.774</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>111</v>
       </c>
@@ -22581,7 +22581,7 @@
         <v>203.72900000000001</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>112</v>
       </c>
@@ -22589,1787 +22589,1675 @@
         <v>202.893</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>22</v>
+        <v>332</v>
       </c>
       <c r="B125">
-        <v>201.83</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+        <v>201.73699999999999</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>332</v>
+        <v>113</v>
       </c>
       <c r="B126">
-        <v>201.73699999999999</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+        <v>201.36699999999999</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B127">
-        <v>201.36699999999999</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+        <v>200.61600000000001</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B128">
-        <v>200.61600000000001</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+        <v>200.11699999999999</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B129">
-        <v>200.11699999999999</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+        <v>199.92400000000001</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B130">
-        <v>199.92400000000001</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+        <v>198.99199999999999</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B131">
-        <v>198.99199999999999</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+        <v>198.72200000000001</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B132">
-        <v>198.72200000000001</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+        <v>196.357</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B133">
-        <v>196.357</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+        <v>195.81800000000001</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B134">
-        <v>195.81800000000001</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+        <v>194.70599999999999</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B135">
-        <v>194.70599999999999</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+        <v>193.15100000000001</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B136">
-        <v>193.15100000000001</v>
-      </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+        <v>191.96700000000001</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B137">
-        <v>191.96700000000001</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+        <v>191.49600000000001</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B138">
-        <v>191.49600000000001</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+        <v>190.64099999999999</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B139">
-        <v>190.64099999999999</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+        <v>190.114</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B140">
-        <v>190.114</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+        <v>189.66399999999999</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B141">
-        <v>189.66399999999999</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+        <v>185.69</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>83</v>
+        <v>129</v>
       </c>
       <c r="B142">
-        <v>187.82300000000001</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+        <v>185.285</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>128</v>
+        <v>333</v>
       </c>
       <c r="B143">
-        <v>185.69</v>
-      </c>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+        <v>183.05600000000001</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B144">
-        <v>185.285</v>
-      </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+        <v>182.797</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>333</v>
+        <v>131</v>
       </c>
       <c r="B145">
-        <v>183.05600000000001</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+        <v>182.65899999999999</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B146">
-        <v>182.797</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+        <v>180.40600000000001</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B147">
-        <v>182.65899999999999</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+        <v>179.32599999999999</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>50</v>
+        <v>134</v>
       </c>
       <c r="B148">
-        <v>180.71</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+        <v>178.786</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B149">
-        <v>180.40600000000001</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+        <v>177.524</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B150">
-        <v>179.32599999999999</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+        <v>176.67500000000001</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B151">
-        <v>178.786</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+        <v>176.578</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B152">
-        <v>177.524</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+        <v>172.36099999999999</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B153">
-        <v>176.67500000000001</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+        <v>170.941</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B154">
-        <v>176.578</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+        <v>170.92400000000001</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B155">
-        <v>172.36099999999999</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+        <v>170.596</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B156">
-        <v>170.941</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+        <v>168.387</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B157">
-        <v>170.92400000000001</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+        <v>167.56399999999999</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B158">
-        <v>170.596</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+        <v>167.42599999999999</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B159">
-        <v>168.387</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+        <v>165.99799999999999</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B160">
-        <v>167.56399999999999</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+        <v>163.304</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B161">
-        <v>167.42599999999999</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+        <v>162.536</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B162">
-        <v>165.99799999999999</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+        <v>161.54</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B163">
-        <v>163.304</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+        <v>160.78299999999999</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B164">
-        <v>162.536</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
+        <v>160.61600000000001</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B165">
-        <v>161.54</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
+        <v>160.46299999999999</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>149</v>
+        <v>334</v>
       </c>
       <c r="B166">
-        <v>160.78299999999999</v>
-      </c>
-    </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.35">
+        <v>159.102</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B167">
-        <v>160.61600000000001</v>
-      </c>
-    </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.35">
+        <v>159.07300000000001</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B168">
-        <v>160.46299999999999</v>
-      </c>
-    </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.35">
+        <v>158.44</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>334</v>
+        <v>154</v>
       </c>
       <c r="B169">
-        <v>159.102</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.35">
+        <v>157.66499999999999</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>152</v>
+        <v>335</v>
       </c>
       <c r="B170">
-        <v>159.07300000000001</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
+        <v>157.05600000000001</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B171">
-        <v>158.44</v>
-      </c>
-    </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.35">
+        <v>156.86799999999999</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B172">
-        <v>157.66499999999999</v>
-      </c>
-    </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.35">
+        <v>156.792</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>335</v>
+        <v>157</v>
       </c>
       <c r="B173">
-        <v>157.05600000000001</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.35">
+        <v>154.37700000000001</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B174">
-        <v>156.86799999999999</v>
-      </c>
-    </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.35">
+        <v>153.124</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B175">
-        <v>156.792</v>
-      </c>
-    </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.35">
+        <v>151.83699999999999</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>38</v>
+        <v>160</v>
       </c>
       <c r="B176">
-        <v>156.75200000000001</v>
-      </c>
-    </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.35">
+        <v>151.59899999999999</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="B177">
-        <v>154.88800000000001</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.35">
+        <v>150.13999999999999</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B178">
-        <v>154.37700000000001</v>
-      </c>
-    </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.35">
+        <v>149.61699999999999</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B179">
-        <v>153.124</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.35">
+        <v>149.035</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B180">
-        <v>151.83699999999999</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.35">
+        <v>148.84700000000001</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B181">
-        <v>151.59899999999999</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.35">
+        <v>148.80799999999999</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B182">
-        <v>150.13999999999999</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.35">
+        <v>148.78200000000001</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B183">
-        <v>149.61699999999999</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.35">
+        <v>148.72</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B184">
-        <v>149.035</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
+        <v>147.96600000000001</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B185">
-        <v>148.84700000000001</v>
-      </c>
-    </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
+        <v>147.48599999999999</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B186">
-        <v>148.80799999999999</v>
-      </c>
-    </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
+        <v>146.68899999999999</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B187">
-        <v>148.78200000000001</v>
-      </c>
-    </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
+        <v>146.608</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B188">
-        <v>148.72</v>
-      </c>
-    </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
+        <v>146.27099999999999</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B189">
-        <v>147.96600000000001</v>
-      </c>
-    </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
+        <v>146.09700000000001</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B190">
-        <v>147.48599999999999</v>
-      </c>
-    </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
+        <v>144.78800000000001</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B191">
-        <v>146.68899999999999</v>
-      </c>
-    </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
+        <v>143.68700000000001</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B192">
-        <v>146.608</v>
-      </c>
-    </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
+        <v>143.24199999999999</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B193">
-        <v>146.27099999999999</v>
-      </c>
-    </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
+        <v>142.023</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B194">
-        <v>146.09700000000001</v>
-      </c>
-    </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
+        <v>141.44900000000001</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B195">
-        <v>144.78800000000001</v>
-      </c>
-    </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
+        <v>140.80799999999999</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B196">
-        <v>143.68700000000001</v>
-      </c>
-    </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
+        <v>140.721</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B197">
-        <v>143.24199999999999</v>
-      </c>
-    </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
+        <v>140.41300000000001</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B198">
-        <v>142.023</v>
-      </c>
-    </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
+        <v>140.054</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>155</v>
+        <v>183</v>
       </c>
       <c r="B199">
-        <v>141.98500000000001</v>
-      </c>
-    </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
+        <v>139.74</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B200">
-        <v>141.44900000000001</v>
-      </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
+        <v>139.57599999999999</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B201">
-        <v>140.80799999999999</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
+        <v>139.13399999999999</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B202">
-        <v>140.721</v>
-      </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.35">
+        <v>138.14400000000001</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B203">
-        <v>140.41300000000001</v>
-      </c>
-    </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.35">
+        <v>137.941</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B204">
-        <v>140.054</v>
-      </c>
-    </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.35">
+        <v>137.904</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B205">
-        <v>139.74</v>
-      </c>
-    </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.35">
+        <v>137.68600000000001</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>184</v>
+        <v>336</v>
       </c>
       <c r="B206">
-        <v>139.57599999999999</v>
-      </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.35">
+        <v>137.596</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B207">
-        <v>139.13399999999999</v>
-      </c>
-    </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.35">
+        <v>137.56200000000001</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B208">
-        <v>138.14400000000001</v>
-      </c>
-    </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.35">
+        <v>136.58799999999999</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B209">
-        <v>137.941</v>
-      </c>
-    </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.35">
+        <v>136.346</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B210">
-        <v>137.904</v>
-      </c>
-    </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.35">
+        <v>136.285</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B211">
-        <v>137.68600000000001</v>
-      </c>
-    </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.35">
+        <v>135.983</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>336</v>
+        <v>195</v>
       </c>
       <c r="B212">
-        <v>137.596</v>
-      </c>
-    </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.35">
+        <v>135.45599999999999</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B213">
-        <v>137.56200000000001</v>
-      </c>
-    </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.35">
+        <v>135.35900000000001</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>162</v>
+        <v>197</v>
       </c>
       <c r="B214">
-        <v>137.19499999999999</v>
-      </c>
-    </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.35">
+        <v>134.34200000000001</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B215">
-        <v>136.58799999999999</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.35">
+        <v>133.13200000000001</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="B216">
-        <v>136.346</v>
-      </c>
-    </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.35">
+        <v>131.01</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B217">
-        <v>136.285</v>
-      </c>
-    </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.35">
+        <v>130.501</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B218">
-        <v>135.983</v>
-      </c>
-    </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.35">
+        <v>129.62</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>195</v>
+        <v>337</v>
       </c>
       <c r="B219">
-        <v>135.45599999999999</v>
-      </c>
-    </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.35">
+        <v>128.691</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="B220">
-        <v>135.35900000000001</v>
-      </c>
-    </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.35">
+        <v>128.023</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B221">
-        <v>134.34200000000001</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.35">
+        <v>127.99299999999999</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B222">
-        <v>133.13200000000001</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" x14ac:dyDescent="0.35">
+        <v>127.744</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="B223">
-        <v>131.01</v>
-      </c>
-    </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.35">
+        <v>127.13800000000001</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="B224">
-        <v>130.9</v>
-      </c>
-    </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.35">
+        <v>126.005</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B225">
-        <v>130.501</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.35">
+        <v>125.77800000000001</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B226">
-        <v>129.62</v>
-      </c>
-    </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.35">
+        <v>125.467</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>337</v>
+        <v>209</v>
       </c>
       <c r="B227">
-        <v>128.691</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.35">
+        <v>125.28400000000001</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="B228">
-        <v>128.023</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.35">
+        <v>124.99</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B229">
-        <v>127.99299999999999</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.35">
+        <v>124.229</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B230">
-        <v>127.744</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.35">
+        <v>124.01600000000001</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="B231">
-        <v>127.13800000000001</v>
-      </c>
-    </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.35">
+        <v>123.47499999999999</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B232">
-        <v>126.005</v>
-      </c>
-    </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.35">
+        <v>122.925</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B233">
-        <v>125.77800000000001</v>
-      </c>
-    </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.35">
+        <v>122.756</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B234">
-        <v>125.467</v>
-      </c>
-    </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.35">
+        <v>122.646</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>209</v>
+        <v>338</v>
       </c>
       <c r="B235">
-        <v>125.28400000000001</v>
-      </c>
-    </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.35">
+        <v>122.28</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B236">
-        <v>124.99</v>
-      </c>
-    </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.35">
+        <v>122.129</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="B237">
-        <v>124.229</v>
-      </c>
-    </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.35">
+        <v>121.873</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="B238">
-        <v>124.01600000000001</v>
-      </c>
-    </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.35">
+        <v>121.749</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>108</v>
+        <v>220</v>
       </c>
       <c r="B239">
-        <v>123.624</v>
-      </c>
-    </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.35">
+        <v>121.629</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B240">
-        <v>123.47499999999999</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.35">
+        <v>121.483</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B241">
-        <v>122.925</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.35">
+        <v>121.18600000000001</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B242">
-        <v>122.756</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.35">
+        <v>120.41800000000001</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="B243">
-        <v>122.646</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.35">
+        <v>119.748</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>338</v>
+        <v>225</v>
       </c>
       <c r="B244">
-        <v>122.28</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.35">
+        <v>118.601</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="B245">
-        <v>122.129</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.35">
+        <v>118.456</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B246">
-        <v>121.873</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.35">
+        <v>118.453</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="B247">
-        <v>121.749</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.35">
+        <v>118.221</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="B248">
-        <v>121.629</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.35">
+        <v>118.18600000000001</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="B249">
-        <v>121.483</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.35">
+        <v>118.104</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="B250">
-        <v>121.18600000000001</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.35">
+        <v>117.35</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="B251">
-        <v>120.41800000000001</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.35">
+        <v>117.041</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="B252">
-        <v>119.748</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.35">
+        <v>116.998</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="B253">
-        <v>118.601</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.35">
+        <v>116.81100000000001</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B254">
-        <v>118.456</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.35">
+        <v>116.688</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="B255">
-        <v>118.453</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.35">
+        <v>116.477</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="B256">
-        <v>118.221</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.35">
+        <v>116.386</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="B257">
-        <v>118.18600000000001</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.35">
+        <v>116.173</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="B258">
-        <v>118.104</v>
-      </c>
-    </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.35">
+        <v>115.908</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="B259">
-        <v>117.35</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.35">
+        <v>115.479</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="B260">
-        <v>117.041</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.35">
+        <v>115.395</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="B261">
-        <v>116.998</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.35">
+        <v>115.30200000000001</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="B262">
-        <v>116.81100000000001</v>
-      </c>
-    </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.35">
+        <v>114.70099999999999</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="B263">
-        <v>116.688</v>
-      </c>
-    </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.35">
+        <v>114.581</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="B264">
-        <v>116.477</v>
-      </c>
-    </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.35">
+        <v>114.363</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="B265">
-        <v>116.386</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.35">
+        <v>114.336</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="B266">
-        <v>116.173</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.35">
+        <v>114.334</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="B267">
-        <v>115.908</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.35">
+        <v>114.288</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="B268">
-        <v>115.479</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.35">
+        <v>113.746</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="B269">
-        <v>115.395</v>
-      </c>
-    </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.35">
+        <v>113.575</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="B270">
-        <v>115.35299999999999</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.35">
+        <v>113.011</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="B271">
-        <v>115.30200000000001</v>
-      </c>
-    </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.35">
+        <v>112.893</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="B272">
-        <v>114.70099999999999</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.35">
+        <v>112.539</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B273">
-        <v>114.581</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.35">
+        <v>112.524</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="B274">
-        <v>114.363</v>
-      </c>
-    </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.35">
+        <v>112.431</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="B275">
-        <v>114.336</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.35">
+        <v>112.21899999999999</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="B276">
-        <v>114.334</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.35">
+        <v>112.05200000000001</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="B277">
-        <v>114.288</v>
-      </c>
-    </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.35">
+        <v>112.003</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="B278">
-        <v>113.746</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.35">
+        <v>111.52</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="B279">
-        <v>113.575</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.35">
+        <v>111.50700000000001</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="B280">
-        <v>113.011</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.35">
+        <v>111.346</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>141</v>
+        <v>263</v>
       </c>
       <c r="B281">
-        <v>112.949</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.35">
+        <v>111.166</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="B282">
-        <v>112.893</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.35">
+        <v>110.337</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>254</v>
+        <v>344</v>
       </c>
       <c r="B283">
-        <v>112.539</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.35">
+        <v>110.002</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B284">
-        <v>112.524</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.35">
+        <v>109.851</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>256</v>
+        <v>343</v>
       </c>
       <c r="B285">
-        <v>112.431</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.35">
+        <v>109.831</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>212</v>
+        <v>266</v>
       </c>
       <c r="B286">
-        <v>112.395</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.35">
+        <v>109.36799999999999</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="B287">
-        <v>112.21899999999999</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.35">
+        <v>109.131</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="B288">
-        <v>112.05200000000001</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.35">
+        <v>108.85299999999999</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="B289">
-        <v>112.003</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.35">
+        <v>108.733</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>116</v>
+        <v>270</v>
       </c>
       <c r="B290">
-        <v>111.696</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.35">
+        <v>108.267</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="B291">
-        <v>111.52</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.35">
+        <v>108.154</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B292">
-        <v>111.50700000000001</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.926</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="B293">
-        <v>111.346</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.92</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="B294">
-        <v>111.166</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.803</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="B295">
-        <v>110.337</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.729</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>344</v>
+        <v>276</v>
       </c>
       <c r="B296">
-        <v>110.002</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.419</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="B297">
-        <v>109.851</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.377</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>343</v>
+        <v>278</v>
       </c>
       <c r="B298">
-        <v>109.831</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.31100000000001</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="B299">
-        <v>109.36799999999999</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.288</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>267</v>
+        <v>339</v>
       </c>
       <c r="B300">
-        <v>109.131</v>
-      </c>
-    </row>
-    <row r="301" spans="1:2" x14ac:dyDescent="0.35">
+        <v>106.101</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B301">
-        <v>108.85299999999999</v>
-      </c>
-    </row>
-    <row r="302" spans="1:2" x14ac:dyDescent="0.35">
+        <v>105.788</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="B302">
-        <v>108.733</v>
-      </c>
-    </row>
-    <row r="303" spans="1:2" x14ac:dyDescent="0.35">
+        <v>105.54300000000001</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="B303">
-        <v>108.267</v>
-      </c>
-    </row>
-    <row r="304" spans="1:2" x14ac:dyDescent="0.35">
+        <v>105.505</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="B304">
-        <v>108.154</v>
-      </c>
-    </row>
-    <row r="305" spans="1:2" x14ac:dyDescent="0.35">
+        <v>104.91800000000001</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="B305">
-        <v>106.926</v>
-      </c>
-    </row>
-    <row r="306" spans="1:2" x14ac:dyDescent="0.35">
+        <v>104.639</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="B306">
-        <v>106.92</v>
-      </c>
-    </row>
-    <row r="307" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.994</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="B307">
-        <v>106.803</v>
-      </c>
-    </row>
-    <row r="308" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.986</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="B308">
-        <v>106.729</v>
-      </c>
-    </row>
-    <row r="309" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.71299999999999</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="B309">
-        <v>106.419</v>
-      </c>
-    </row>
-    <row r="310" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.60599999999999</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="B310">
-        <v>106.377</v>
-      </c>
-    </row>
-    <row r="311" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.559</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="B311">
-        <v>106.31100000000001</v>
-      </c>
-    </row>
-    <row r="312" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.533</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="B312">
-        <v>106.288</v>
-      </c>
-    </row>
-    <row r="313" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.489</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>339</v>
+        <v>292</v>
       </c>
       <c r="B313">
-        <v>106.101</v>
-      </c>
-    </row>
-    <row r="314" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.434</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="B314">
-        <v>105.788</v>
-      </c>
-    </row>
-    <row r="315" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.291</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>281</v>
+        <v>340</v>
       </c>
       <c r="B315">
-        <v>105.54300000000001</v>
-      </c>
-    </row>
-    <row r="316" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.105</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="B316">
-        <v>105.505</v>
-      </c>
-    </row>
-    <row r="317" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103.006</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="B317">
-        <v>104.91800000000001</v>
-      </c>
-    </row>
-    <row r="318" spans="1:2" x14ac:dyDescent="0.35">
+        <v>102.911</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="B318">
-        <v>104.639</v>
-      </c>
-    </row>
-    <row r="319" spans="1:2" x14ac:dyDescent="0.35">
+        <v>102.774</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="B319">
-        <v>103.994</v>
-      </c>
-    </row>
-    <row r="320" spans="1:2" x14ac:dyDescent="0.35">
+        <v>102.372</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="B320">
-        <v>103.986</v>
-      </c>
-    </row>
-    <row r="321" spans="1:2" x14ac:dyDescent="0.35">
+        <v>102.238</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="B321">
-        <v>103.71299999999999</v>
-      </c>
-    </row>
-    <row r="322" spans="1:2" x14ac:dyDescent="0.35">
+        <v>101.836</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="B322">
-        <v>103.60599999999999</v>
-      </c>
-    </row>
-    <row r="323" spans="1:2" x14ac:dyDescent="0.35">
+        <v>101.41800000000001</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>289</v>
+        <v>341</v>
       </c>
       <c r="B323">
-        <v>103.559</v>
-      </c>
-    </row>
-    <row r="324" spans="1:2" x14ac:dyDescent="0.35">
+        <v>101.35899999999999</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="B324">
-        <v>103.533</v>
-      </c>
-    </row>
-    <row r="325" spans="1:2" x14ac:dyDescent="0.35">
+        <v>101.34399999999999</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>291</v>
+        <v>302</v>
       </c>
       <c r="B325">
-        <v>103.489</v>
-      </c>
-    </row>
-    <row r="326" spans="1:2" x14ac:dyDescent="0.35">
+        <v>101.318</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="B326">
-        <v>103.434</v>
-      </c>
-    </row>
-    <row r="327" spans="1:2" x14ac:dyDescent="0.35">
+        <v>101.31699999999999</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="B327">
-        <v>103.291</v>
-      </c>
-    </row>
-    <row r="328" spans="1:2" x14ac:dyDescent="0.35">
+        <v>100.938</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>105</v>
+        <v>305</v>
       </c>
       <c r="B328">
-        <v>103.134</v>
-      </c>
-    </row>
-    <row r="329" spans="1:2" x14ac:dyDescent="0.35">
+        <v>100.694</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>340</v>
+        <v>306</v>
       </c>
       <c r="B329">
-        <v>103.105</v>
-      </c>
-    </row>
-    <row r="330" spans="1:2" x14ac:dyDescent="0.35">
+        <v>100.51300000000001</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="B330">
-        <v>103.006</v>
-      </c>
-    </row>
-    <row r="331" spans="1:2" x14ac:dyDescent="0.35">
+        <v>100.252</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="B331">
-        <v>102.911</v>
-      </c>
-    </row>
-    <row r="332" spans="1:2" x14ac:dyDescent="0.35">
+        <v>100.15900000000001</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="B332">
-        <v>102.774</v>
-      </c>
-    </row>
-    <row r="333" spans="1:2" x14ac:dyDescent="0.35">
+        <v>100.136</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="B333">
-        <v>102.372</v>
-      </c>
-    </row>
-    <row r="334" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A334" t="s">
-        <v>298</v>
-      </c>
-      <c r="B334">
-        <v>102.238</v>
-      </c>
-    </row>
-    <row r="335" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A335" t="s">
-        <v>299</v>
-      </c>
-      <c r="B335">
-        <v>101.836</v>
-      </c>
-    </row>
-    <row r="336" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A336" t="s">
-        <v>300</v>
-      </c>
-      <c r="B336">
-        <v>101.41800000000001</v>
-      </c>
-    </row>
-    <row r="337" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A337" t="s">
-        <v>341</v>
-      </c>
-      <c r="B337">
-        <v>101.35899999999999</v>
-      </c>
-    </row>
-    <row r="338" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A338" t="s">
-        <v>301</v>
-      </c>
-      <c r="B338">
-        <v>101.34399999999999</v>
-      </c>
-    </row>
-    <row r="339" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A339" t="s">
-        <v>302</v>
-      </c>
-      <c r="B339">
-        <v>101.318</v>
-      </c>
-    </row>
-    <row r="340" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A340" t="s">
-        <v>303</v>
-      </c>
-      <c r="B340">
-        <v>101.31699999999999</v>
-      </c>
-    </row>
-    <row r="341" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A341" t="s">
-        <v>304</v>
-      </c>
-      <c r="B341">
-        <v>100.938</v>
-      </c>
-    </row>
-    <row r="342" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A342" t="s">
-        <v>305</v>
-      </c>
-      <c r="B342">
-        <v>100.694</v>
-      </c>
-    </row>
-    <row r="343" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A343" t="s">
-        <v>306</v>
-      </c>
-      <c r="B343">
-        <v>100.51300000000001</v>
-      </c>
-    </row>
-    <row r="344" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A344" t="s">
-        <v>307</v>
-      </c>
-      <c r="B344">
-        <v>100.252</v>
-      </c>
-    </row>
-    <row r="345" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A345" t="s">
-        <v>308</v>
-      </c>
-      <c r="B345">
-        <v>100.15900000000001</v>
-      </c>
-    </row>
-    <row r="346" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A346" t="s">
-        <v>309</v>
-      </c>
-      <c r="B346">
-        <v>100.136</v>
-      </c>
-    </row>
-    <row r="347" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A347" t="s">
-        <v>310</v>
-      </c>
-      <c r="B347">
         <v>100.128</v>
       </c>
     </row>
@@ -24477,216 +24365,205 @@
     <hyperlink ref="A122" r:id="rId100" tooltip="Little Rock, Arkansas" display="https://en.wikipedia.org/wiki/Little_Rock,_Arkansas" xr:uid="{B5BA475A-0115-4D86-96AE-B12DA1AE4B50}"/>
     <hyperlink ref="A123" r:id="rId101" tooltip="Amarillo, Texas" display="https://en.wikipedia.org/wiki/Amarillo,_Texas" xr:uid="{A4B3D8CF-3157-43C5-BD2A-77C10D18D5C7}"/>
     <hyperlink ref="A124" r:id="rId102" tooltip="Overland Park, Kansas" display="https://en.wikipedia.org/wiki/Overland_Park,_Kansas" xr:uid="{757F326E-75D1-49D0-AA50-C283BF7E0555}"/>
-    <hyperlink ref="A127" r:id="rId103" tooltip="Mobile, Alabama" display="https://en.wikipedia.org/wiki/Mobile,_Alabama" xr:uid="{4E2896C7-D20A-4C4D-80BA-6FA7EE84347E}"/>
-    <hyperlink ref="A128" r:id="rId104" tooltip="Oxnard, California" display="https://en.wikipedia.org/wiki/Oxnard,_California" xr:uid="{052FB3E4-9739-4330-B5B5-9CD746CCCA7E}"/>
-    <hyperlink ref="A129" r:id="rId105" tooltip="Grand Rapids, Michigan" display="https://en.wikipedia.org/wiki/Grand_Rapids,_Michigan" xr:uid="{8D0C128B-FFDC-481C-A82A-2478374C7FFC}"/>
-    <hyperlink ref="A130" r:id="rId106" tooltip="Peoria, Arizona" display="https://en.wikipedia.org/wiki/Peoria,_Arizona" xr:uid="{42DE2250-B81C-4119-B875-3B3D2BBC0774}"/>
-    <hyperlink ref="A131" r:id="rId107" tooltip="Vancouver, Washington" display="https://en.wikipedia.org/wiki/Vancouver,_Washington" xr:uid="{56DB179A-8427-415C-820F-20758DEF26F4}"/>
-    <hyperlink ref="A132" r:id="rId108" tooltip="Knoxville, Tennessee" display="https://en.wikipedia.org/wiki/Knoxville,_Tennessee" xr:uid="{3191FCC6-6BD4-4A6D-AC10-B7329A152ABD}"/>
-    <hyperlink ref="A133" r:id="rId109" tooltip="Birmingham, Alabama" display="https://en.wikipedia.org/wiki/Birmingham,_Alabama" xr:uid="{B0F1434B-2180-4728-BBB7-DC5D157943C1}"/>
-    <hyperlink ref="A134" r:id="rId110" tooltip="Montgomery, Alabama" display="https://en.wikipedia.org/wiki/Montgomery,_Alabama" xr:uid="{243C3328-7F74-4607-A5BF-0DB07F7695E3}"/>
-    <hyperlink ref="A135" r:id="rId111" tooltip="Providence, Rhode Island" display="https://en.wikipedia.org/wiki/Providence,_Rhode_Island" xr:uid="{B18F437D-0BD6-49A0-B395-48E8ACF5A67A}"/>
-    <hyperlink ref="A136" r:id="rId112" tooltip="Huntington Beach, California" display="https://en.wikipedia.org/wiki/Huntington_Beach,_California" xr:uid="{EC38142B-2562-4B33-A90A-23AA220C0C86}"/>
-    <hyperlink ref="A137" r:id="rId113" tooltip="Brownsville, Texas" display="https://en.wikipedia.org/wiki/Brownsville,_Texas" xr:uid="{C7CAF846-2A11-42FE-8CCC-19177CAE3C57}"/>
-    <hyperlink ref="A138" r:id="rId114" tooltip="Chattanooga, Tennessee" display="https://en.wikipedia.org/wiki/Chattanooga,_Tennessee" xr:uid="{7DD8093A-1E37-4F1C-96D2-248C52349C1E}"/>
-    <hyperlink ref="A139" r:id="rId115" tooltip="Fort Lauderdale, Florida" display="https://en.wikipedia.org/wiki/Fort_Lauderdale,_Florida" xr:uid="{228D6E06-E1E1-40D8-8D34-B05A4AF7959C}"/>
-    <hyperlink ref="A140" r:id="rId116" tooltip="Tempe, Arizona" display="https://en.wikipedia.org/wiki/Tempe,_Arizona" xr:uid="{9A6B5A9C-D0F6-446D-9C4E-67078BB98A2E}"/>
-    <hyperlink ref="A141" r:id="rId117" tooltip="Akron, Ohio" display="https://en.wikipedia.org/wiki/Akron,_Ohio" xr:uid="{819F738E-195E-463F-AB6B-389E157E76F2}"/>
-    <hyperlink ref="A142" r:id="rId118" tooltip="Glendale, California" display="https://en.wikipedia.org/wiki/Glendale,_California" xr:uid="{47C7DBF0-2015-4291-83B3-91C482756D97}"/>
-    <hyperlink ref="A143" r:id="rId119" tooltip="Clarksville, Tennessee" display="https://en.wikipedia.org/wiki/Clarksville,_Tennessee" xr:uid="{60A80EAF-F3C7-408C-A885-091C7F98C21C}"/>
-    <hyperlink ref="A144" r:id="rId120" tooltip="Ontario, California" display="https://en.wikipedia.org/wiki/Ontario,_California" xr:uid="{5ADAA54E-67DF-4A47-A555-F8A040679E6E}"/>
-    <hyperlink ref="A146" r:id="rId121" tooltip="Elk Grove, California" display="https://en.wikipedia.org/wiki/Elk_Grove,_California" xr:uid="{7D8A5CB7-CE45-47B5-9BA9-EC23CD3121FC}"/>
-    <hyperlink ref="A147" r:id="rId122" tooltip="Cary, North Carolina" display="https://en.wikipedia.org/wiki/Cary,_North_Carolina" xr:uid="{79238080-FBEB-413C-B4EC-25113F093DAB}"/>
-    <hyperlink ref="A148" r:id="rId123" tooltip="Aurora, Illinois" display="https://en.wikipedia.org/wiki/Aurora,_Illinois" xr:uid="{7763C6BE-7E5F-45AC-83AE-A0467F43B551}"/>
-    <hyperlink ref="A149" r:id="rId124" tooltip="Salem, Oregon" display="https://en.wikipedia.org/wiki/Salem,_Oregon" xr:uid="{57C4AD57-3BE4-4858-B3CE-4383A20849AE}"/>
-    <hyperlink ref="A150" r:id="rId125" tooltip="Pembroke Pines, Florida" display="https://en.wikipedia.org/wiki/Pembroke_Pines,_Florida" xr:uid="{5504AF73-E1C8-496D-9493-736EDFDEB61C}"/>
-    <hyperlink ref="A151" r:id="rId126" tooltip="Eugene, Oregon" display="https://en.wikipedia.org/wiki/Eugene,_Oregon" xr:uid="{3CC9226D-8DBF-4F8F-A94B-21C0F2968F0D}"/>
-    <hyperlink ref="A152" r:id="rId127" tooltip="Santa Rosa, California" display="https://en.wikipedia.org/wiki/Santa_Rosa,_California" xr:uid="{A9BBF8A8-C94B-4BA8-A909-D6DAB891141D}"/>
-    <hyperlink ref="A153" r:id="rId128" tooltip="Rancho Cucamonga, California" display="https://en.wikipedia.org/wiki/Rancho_Cucamonga,_California" xr:uid="{920CC947-E031-4EB0-986D-9A97014345D7}"/>
-    <hyperlink ref="A154" r:id="rId129" tooltip="Shreveport, Louisiana" display="https://en.wikipedia.org/wiki/Shreveport,_Louisiana" xr:uid="{C4A0CDD8-B0FF-4BDA-981D-6A3CE676142A}"/>
-    <hyperlink ref="A155" r:id="rId130" tooltip="Garden Grove, California" display="https://en.wikipedia.org/wiki/Garden_Grove,_California" xr:uid="{A54A8506-CC2D-4453-9241-07C4C35486A9}"/>
-    <hyperlink ref="A156" r:id="rId131" tooltip="Oceanside, California" display="https://en.wikipedia.org/wiki/Oceanside,_California" xr:uid="{B5E0D532-AA0F-4F4A-B48A-DDB52F59614B}"/>
-    <hyperlink ref="A157" r:id="rId132" tooltip="Fort Collins, Colorado" display="https://en.wikipedia.org/wiki/Fort_Collins,_Colorado" xr:uid="{48526A50-3DE3-4820-B7FC-1F8EA26E1FF1}"/>
-    <hyperlink ref="A158" r:id="rId133" tooltip="Springfield, Missouri" display="https://en.wikipedia.org/wiki/Springfield,_Missouri" xr:uid="{159962FC-4A24-49B3-939A-BF554AD8F9CE}"/>
-    <hyperlink ref="A159" r:id="rId134" tooltip="Murfreesboro, Tennessee" display="https://en.wikipedia.org/wiki/Murfreesboro,_Tennessee" xr:uid="{028986A8-13D8-45DB-8308-38F5D6975394}"/>
-    <hyperlink ref="A160" r:id="rId135" tooltip="Surprise, Arizona" display="https://en.wikipedia.org/wiki/Surprise,_Arizona" xr:uid="{9F81C077-8E62-4CE0-B2F1-3D8ED9546E89}"/>
-    <hyperlink ref="A161" r:id="rId136" tooltip="Lancaster, California" display="https://en.wikipedia.org/wiki/Lancaster,_California" xr:uid="{BA04C0C3-2052-4003-A556-BE985789E293}"/>
-    <hyperlink ref="A162" r:id="rId137" tooltip="Denton, Texas" display="https://en.wikipedia.org/wiki/Denton,_Texas" xr:uid="{C4DEA4D8-6231-44D9-BE26-5A855CCEE36D}"/>
-    <hyperlink ref="A163" r:id="rId138" tooltip="Roseville, California" display="https://en.wikipedia.org/wiki/Roseville,_California" xr:uid="{AB952918-E34D-40D6-8C85-3CC456F7EEE4}"/>
-    <hyperlink ref="A164" r:id="rId139" tooltip="Palmdale, California" display="https://en.wikipedia.org/wiki/Palmdale,_California" xr:uid="{5D4C2C43-9935-4AF9-A0A2-B3546E301F66}"/>
-    <hyperlink ref="A165" r:id="rId140" tooltip="Corona, California" display="https://en.wikipedia.org/wiki/Corona,_California" xr:uid="{79F07F89-247B-4564-B1CF-63DA0443AD2D}"/>
-    <hyperlink ref="A166" r:id="rId141" tooltip="Salinas, California" display="https://en.wikipedia.org/wiki/Salinas,_California" xr:uid="{0A5A2FD9-D666-4D98-8976-B306D0B0C5E2}"/>
-    <hyperlink ref="A167" r:id="rId142" tooltip="Killeen, Texas" display="https://en.wikipedia.org/wiki/Killeen,_Texas" xr:uid="{9DF4AF29-351F-4CA2-9882-62B0E04705C0}"/>
-    <hyperlink ref="A168" r:id="rId143" tooltip="Paterson, New Jersey" display="https://en.wikipedia.org/wiki/Paterson,_New_Jersey" xr:uid="{030A6D78-319E-4361-81DF-9FA91B5F8363}"/>
-    <hyperlink ref="A170" r:id="rId144" tooltip="Hollywood, Florida" display="https://en.wikipedia.org/wiki/Hollywood,_Florida" xr:uid="{2E514F97-08AE-4C83-8AA5-249046DF2182}"/>
-    <hyperlink ref="A171" r:id="rId145" tooltip="Hayward, California" display="https://en.wikipedia.org/wiki/Hayward,_California" xr:uid="{758E4979-EA25-41AD-9A83-DAE7CABC51CB}"/>
-    <hyperlink ref="A172" r:id="rId146" tooltip="Charleston, South Carolina" display="https://en.wikipedia.org/wiki/Charleston,_South_Carolina" xr:uid="{ABF30A89-881F-4D1E-A027-BD2DF9FA7396}"/>
-    <hyperlink ref="A174" r:id="rId147" tooltip="Lakewood, Colorado" display="https://en.wikipedia.org/wiki/Lakewood,_Colorado" xr:uid="{D4B8E640-228C-40FA-A462-8570AB31B310}"/>
-    <hyperlink ref="A175" r:id="rId148" tooltip="Sunnyvale, California" display="https://en.wikipedia.org/wiki/Sunnyvale,_California" xr:uid="{868F929C-5F4D-4AA9-9644-AA6FAFE84F3F}"/>
-    <hyperlink ref="A177" r:id="rId149" tooltip="Springfield, Massachusetts" display="https://en.wikipedia.org/wiki/Springfield,_Massachusetts" xr:uid="{5195277A-6E96-47B6-8014-5C525CB7A9A9}"/>
-    <hyperlink ref="A178" r:id="rId150" tooltip="Bellevue, Washington" display="https://en.wikipedia.org/wiki/Bellevue,_Washington" xr:uid="{6F9C2962-8946-46D9-A375-62E5C91270D7}"/>
-    <hyperlink ref="A179" r:id="rId151" tooltip="Naperville, Illinois" display="https://en.wikipedia.org/wiki/Naperville,_Illinois" xr:uid="{4DB54CD8-BD51-4D4C-9FD1-30ECAFA73408}"/>
-    <hyperlink ref="A180" r:id="rId152" tooltip="Joliet, Illinois" display="https://en.wikipedia.org/wiki/Joliet,_Illinois" xr:uid="{2B68DF39-77FA-4587-91BC-440C7E1FAEA9}"/>
-    <hyperlink ref="A181" r:id="rId153" tooltip="Bridgeport, Connecticut" display="https://en.wikipedia.org/wiki/Bridgeport,_Connecticut" xr:uid="{6C639E49-E2CF-43E5-A98A-E0DB9579406B}"/>
-    <hyperlink ref="A182" r:id="rId154" tooltip="Mesquite, Texas" display="https://en.wikipedia.org/wiki/Mesquite,_Texas" xr:uid="{95F60B5B-76CA-456E-8F1E-9C9BBDB8D150}"/>
-    <hyperlink ref="A183" r:id="rId155" tooltip="Pasadena, Texas" display="https://en.wikipedia.org/wiki/Pasadena,_Texas" xr:uid="{59E07B82-9CBF-494B-9C62-E014257ECB57}"/>
-    <hyperlink ref="A184" r:id="rId156" tooltip="Olathe, Kansas" display="https://en.wikipedia.org/wiki/Olathe,_Kansas" xr:uid="{8A551723-EC13-4EAC-A759-3831FCDE0FBA}"/>
-    <hyperlink ref="A185" r:id="rId157" tooltip="Escondido, California" display="https://en.wikipedia.org/wiki/Escondido,_California" xr:uid="{7C50450E-C974-44E4-B1DD-C67F306B77D9}"/>
-    <hyperlink ref="A186" r:id="rId158" tooltip="Savannah, Georgia" display="https://en.wikipedia.org/wiki/Savannah,_Georgia" xr:uid="{B437D653-1143-4A10-BADC-D286B6ACC723}"/>
-    <hyperlink ref="A187" r:id="rId159" tooltip="McAllen, Texas" display="https://en.wikipedia.org/wiki/McAllen,_Texas" xr:uid="{AEC35262-3478-445B-84D6-751CD4AB3EB8}"/>
-    <hyperlink ref="A188" r:id="rId160" tooltip="Gainesville, Florida" display="https://en.wikipedia.org/wiki/Gainesville,_Florida" xr:uid="{515430DE-7083-474C-B331-11441A93126F}"/>
-    <hyperlink ref="A189" r:id="rId161" tooltip="Pomona, California" display="https://en.wikipedia.org/wiki/Pomona,_California" xr:uid="{B1094DCC-91EE-4D42-93BC-775D727B4BFB}"/>
-    <hyperlink ref="A190" r:id="rId162" tooltip="Rockford, Illinois" display="https://en.wikipedia.org/wiki/Rockford,_Illinois" xr:uid="{6D481027-4AFF-44F2-88E1-76967CC0E2A6}"/>
-    <hyperlink ref="A191" r:id="rId163" tooltip="Thornton, Colorado" display="https://en.wikipedia.org/wiki/Thornton,_Colorado" xr:uid="{089AD7E4-304F-45D7-8568-F69C04962229}"/>
-    <hyperlink ref="A192" r:id="rId164" tooltip="Waco, Texas" display="https://en.wikipedia.org/wiki/Waco,_Texas" xr:uid="{E2E37336-2BFF-4BA9-B2E9-2AB8AA0B9AA8}"/>
-    <hyperlink ref="A193" r:id="rId165" tooltip="Visalia, California" display="https://en.wikipedia.org/wiki/Visalia,_California" xr:uid="{29E9B44C-BD44-4415-8353-32105E42888C}"/>
-    <hyperlink ref="A194" r:id="rId166" tooltip="Syracuse, New York" display="https://en.wikipedia.org/wiki/Syracuse,_New_York" xr:uid="{A14C8F93-A81F-4C3D-88E4-2AFE1705D539}"/>
-    <hyperlink ref="A195" r:id="rId167" tooltip="Columbia, South Carolina" display="https://en.wikipedia.org/wiki/Columbia,_South_Carolina" xr:uid="{F4F498F5-0B13-4FF8-A95C-1AA4467DE7C6}"/>
-    <hyperlink ref="A196" r:id="rId168" tooltip="Midland, Texas" display="https://en.wikipedia.org/wiki/Midland,_Texas" xr:uid="{E582A898-E936-4550-A605-650D12038D6D}"/>
-    <hyperlink ref="A197" r:id="rId169" tooltip="Miramar, Florida" display="https://en.wikipedia.org/wiki/Miramar,_Florida" xr:uid="{3BA09F94-2888-4164-BE2A-0AF6F7D7563B}"/>
-    <hyperlink ref="A198" r:id="rId170" tooltip="Palm Bay, Florida" display="https://en.wikipedia.org/wiki/Palm_Bay,_Florida" xr:uid="{7AB8CBCA-ACE3-4F96-97A6-330084EF6E97}"/>
-    <hyperlink ref="A200" r:id="rId171" tooltip="Jackson, Mississippi" display="https://en.wikipedia.org/wiki/Jackson,_Mississippi" xr:uid="{452C5DBB-23EC-47E7-8022-C74105F4066E}"/>
-    <hyperlink ref="A201" r:id="rId172" tooltip="Coral Springs, Florida" display="https://en.wikipedia.org/wiki/Coral_Springs,_Florida" xr:uid="{1E574227-B848-43C2-B9F4-22D0F218B4C4}"/>
-    <hyperlink ref="A202" r:id="rId173" tooltip="Victorville, California" display="https://en.wikipedia.org/wiki/Victorville,_California" xr:uid="{52E5C233-3B9B-4865-A502-6B8E7389212C}"/>
-    <hyperlink ref="A203" r:id="rId174" tooltip="Elizabeth, New Jersey" display="https://en.wikipedia.org/wiki/Elizabeth,_New_Jersey" xr:uid="{C8F9B792-D568-48D5-8A78-2D781C24AF74}"/>
-    <hyperlink ref="A204" r:id="rId175" tooltip="Fullerton, California" display="https://en.wikipedia.org/wiki/Fullerton,_California" xr:uid="{5CBFCC65-14FB-4A2B-8F31-F6946EB55A5C}"/>
-    <hyperlink ref="A205" r:id="rId176" tooltip="Meridian, Idaho" display="https://en.wikipedia.org/wiki/Meridian,_Idaho" xr:uid="{597815BB-8ED0-4939-BF0A-55F4A5E8BC50}"/>
-    <hyperlink ref="A206" r:id="rId177" tooltip="Torrance, California" display="https://en.wikipedia.org/wiki/Torrance,_California" xr:uid="{FF8E2C05-3A0A-4C12-A1C2-C8DDF230745D}"/>
-    <hyperlink ref="A207" r:id="rId178" tooltip="Stamford, Connecticut" display="https://en.wikipedia.org/wiki/Stamford,_Connecticut" xr:uid="{03D2E1BE-0681-44F9-BDC4-01AC870E7E56}"/>
-    <hyperlink ref="A208" r:id="rId179" tooltip="West Valley City, Utah" display="https://en.wikipedia.org/wiki/West_Valley_City,_Utah" xr:uid="{13121615-27BF-4675-A1A6-EAD51C7BD23C}"/>
-    <hyperlink ref="A209" r:id="rId180" tooltip="Orange, California" display="https://en.wikipedia.org/wiki/Orange,_California" xr:uid="{4E6A91BB-9161-49ED-B5BE-6E6167F3E176}"/>
-    <hyperlink ref="A210" r:id="rId181" tooltip="Cedar Rapids, Iowa" display="https://en.wikipedia.org/wiki/Cedar_Rapids,_Iowa" xr:uid="{FEA38046-A2F4-4386-B26C-19A067C94BC4}"/>
-    <hyperlink ref="A211" r:id="rId182" tooltip="Warren, Michigan" display="https://en.wikipedia.org/wiki/Warren,_Michigan" xr:uid="{50A9F933-1332-4090-83DE-72B53CE9FAA0}"/>
-    <hyperlink ref="A213" r:id="rId183" tooltip="New Haven, Connecticut" display="https://en.wikipedia.org/wiki/New_Haven,_Connecticut" xr:uid="{36736AE9-BC59-4B0E-9277-4D6FBE835464}"/>
-    <hyperlink ref="A214" r:id="rId184" tooltip="Pasadena, California" display="https://en.wikipedia.org/wiki/Pasadena,_California" xr:uid="{74396265-8002-43E0-9DCC-801960BE01CC}"/>
-    <hyperlink ref="A215" r:id="rId185" tooltip="Kent, Washington" display="https://en.wikipedia.org/wiki/Kent,_Washington" xr:uid="{D5AFC1CD-5101-45C9-AAE5-F44865689E1B}"/>
-    <hyperlink ref="A216" r:id="rId186" tooltip="Dayton, Ohio" display="https://en.wikipedia.org/wiki/Dayton,_Ohio" xr:uid="{31F02388-BE9C-4CE9-97DC-EB6DA4199D2A}"/>
-    <hyperlink ref="A217" r:id="rId187" tooltip="Fargo, North Dakota" display="https://en.wikipedia.org/wiki/Fargo,_North_Dakota" xr:uid="{5386272E-280B-4D18-BA96-A85462C4CCC5}"/>
-    <hyperlink ref="A218" r:id="rId188" tooltip="Lewisville, Texas" display="https://en.wikipedia.org/wiki/Lewisville,_Texas" xr:uid="{7C126BE8-F9E1-4A95-A740-3E8BA349158C}"/>
-    <hyperlink ref="A219" r:id="rId189" tooltip="Carrollton, Texas" display="https://en.wikipedia.org/wiki/Carrollton,_Texas" xr:uid="{D3E15712-3D89-45D0-8D02-1E2E8A00C100}"/>
-    <hyperlink ref="A220" r:id="rId190" tooltip="Round Rock, Texas" display="https://en.wikipedia.org/wiki/Round_Rock,_Texas" xr:uid="{38E0BC55-C7D0-40C4-ACE0-DC353CAEC1E3}"/>
-    <hyperlink ref="A221" r:id="rId191" tooltip="Sterling Heights, Michigan" display="https://en.wikipedia.org/wiki/Sterling_Heights,_Michigan" xr:uid="{17296518-C7F4-4A39-A607-C824D9035787}"/>
-    <hyperlink ref="A222" r:id="rId192" tooltip="Santa Clara, California" display="https://en.wikipedia.org/wiki/Santa_Clara,_California" xr:uid="{0D94D9D7-10A1-4806-80E2-ACF89B9B6747}"/>
-    <hyperlink ref="A223" r:id="rId193" tooltip="Norman, Oklahoma" display="https://en.wikipedia.org/wiki/Norman,_Oklahoma" xr:uid="{C6B26389-B925-4CB9-AA91-0E298A1FADDD}"/>
-    <hyperlink ref="A224" r:id="rId194" tooltip="Columbia, Missouri" display="https://en.wikipedia.org/wiki/Columbia,_Missouri" xr:uid="{0ADE51F5-9EBA-4120-83F6-EBD3A58E90D7}"/>
-    <hyperlink ref="A225" r:id="rId195" tooltip="Abilene, Texas" display="https://en.wikipedia.org/wiki/Abilene,_Texas" xr:uid="{E7C4729C-2C7E-43E8-A6AD-FCC3664ED9A4}"/>
-    <hyperlink ref="A226" r:id="rId196" tooltip="Pearland, Texas" display="https://en.wikipedia.org/wiki/Pearland,_Texas" xr:uid="{9DC3AF36-1C01-4B23-A2FA-5104C8021675}"/>
-    <hyperlink ref="A228" r:id="rId197" tooltip="College Station, Texas" display="https://en.wikipedia.org/wiki/College_Station,_Texas" xr:uid="{D8B084A5-B93D-47A7-8C98-4665850B0F18}"/>
-    <hyperlink ref="A229" r:id="rId198" tooltip="Clovis, California" display="https://en.wikipedia.org/wiki/Clovis,_California" xr:uid="{A5744F83-7207-461E-AAEC-2800B018D389}"/>
-    <hyperlink ref="A230" r:id="rId199" tooltip="West Palm Beach, Florida" display="https://en.wikipedia.org/wiki/West_Palm_Beach,_Florida" xr:uid="{7E4D65CA-0099-4770-8A50-4F4084FAB89E}"/>
-    <hyperlink ref="A231" r:id="rId200" tooltip="Allentown, Pennsylvania" display="https://en.wikipedia.org/wiki/Allentown,_Pennsylvania" xr:uid="{393395BF-6D30-4ED7-BCEE-D1A0798D0761}"/>
-    <hyperlink ref="A232" r:id="rId201" tooltip="North Charleston, South Carolina" display="https://en.wikipedia.org/wiki/North_Charleston,_South_Carolina" xr:uid="{584C8E92-DCE9-4485-B244-A631B2CC3A9C}"/>
-    <hyperlink ref="A233" r:id="rId202" tooltip="Simi Valley, California" display="https://en.wikipedia.org/wiki/Simi_Valley,_California" xr:uid="{829C49A5-275F-478F-AE5B-4EAB3642A1D6}"/>
-    <hyperlink ref="A234" r:id="rId203" tooltip="Topeka, Kansas" display="https://en.wikipedia.org/wiki/Topeka,_Kansas" xr:uid="{67481949-F882-464A-B6A6-626D32A82D50}"/>
-    <hyperlink ref="A235" r:id="rId204" tooltip="Wilmington, North Carolina" display="https://en.wikipedia.org/wiki/Wilmington,_North_Carolina" xr:uid="{2119452B-13EF-4892-9F66-943906FC84DF}"/>
-    <hyperlink ref="A236" r:id="rId205" tooltip="Lakeland, Florida" display="https://en.wikipedia.org/wiki/Lakeland,_Florida" xr:uid="{A1D87FDC-D554-48AC-995A-F6860FBD033E}"/>
-    <hyperlink ref="A237" r:id="rId206" tooltip="Thousand Oaks, California" display="https://en.wikipedia.org/wiki/Thousand_Oaks,_California" xr:uid="{603BAD32-8E4C-4D79-9C8D-5D0954FF0E9F}"/>
-    <hyperlink ref="A238" r:id="rId207" tooltip="Concord, California" display="https://en.wikipedia.org/wiki/Concord,_California" xr:uid="{ED78F782-2868-4B6D-BEDF-A272685AE35D}"/>
-    <hyperlink ref="A239" r:id="rId208" tooltip="Rochester, Minnesota" display="https://en.wikipedia.org/wiki/Rochester,_Minnesota" xr:uid="{D55EE569-B003-47C7-9FB1-2F9EA27369A6}"/>
-    <hyperlink ref="A240" r:id="rId209" tooltip="Vallejo, California" display="https://en.wikipedia.org/wiki/Vallejo,_California" xr:uid="{7097017F-CF66-4243-B160-CF19DE3A2267}"/>
-    <hyperlink ref="A241" r:id="rId210" tooltip="Ann Arbor, Michigan" display="https://en.wikipedia.org/wiki/Ann_Arbor,_Michigan" xr:uid="{553E315B-35D3-44A6-A013-F1E8A0373A52}"/>
-    <hyperlink ref="A242" r:id="rId211" tooltip="Broken Arrow, Oklahoma" display="https://en.wikipedia.org/wiki/Broken_Arrow,_Oklahoma" xr:uid="{0059EE80-8A45-4D03-923A-B99BB1DF140D}"/>
-    <hyperlink ref="A243" r:id="rId212" tooltip="Fairfield, California" display="https://en.wikipedia.org/wiki/Fairfield,_California" xr:uid="{AFA3C10B-D1BB-4925-AA49-774FA576A43D}"/>
-    <hyperlink ref="A245" r:id="rId213" tooltip="Hartford, Connecticut" display="https://en.wikipedia.org/wiki/Hartford,_Connecticut" xr:uid="{1CF83A0B-54E4-4DFB-8F78-8220F113FE27}"/>
-    <hyperlink ref="A246" r:id="rId214" tooltip="Arvada, Colorado" display="https://en.wikipedia.org/wiki/Arvada,_Colorado" xr:uid="{E34E7BC9-DB14-4DC6-A62B-652BB8DC4F39}"/>
-    <hyperlink ref="A247" r:id="rId215" tooltip="Berkeley, California" display="https://en.wikipedia.org/wiki/Berkeley,_California" xr:uid="{F58A1B3A-1363-4070-A1DB-53CD2D8EA801}"/>
-    <hyperlink ref="A248" r:id="rId216" tooltip="Independence, Missouri" display="https://en.wikipedia.org/wiki/Independence,_Missouri" xr:uid="{9552DC8D-5E58-445D-8F54-557CAF5DC4F3}"/>
-    <hyperlink ref="A249" r:id="rId217" tooltip="Billings, Montana" display="https://en.wikipedia.org/wiki/Billings,_Montana" xr:uid="{CAC8EE67-B509-4FDF-B7F0-3C9C0015A709}"/>
-    <hyperlink ref="A250" r:id="rId218" tooltip="Cambridge, Massachusetts" display="https://en.wikipedia.org/wiki/Cambridge,_Massachusetts" xr:uid="{B6C026EF-7901-4ADD-AB65-B069FF3C8C5E}"/>
-    <hyperlink ref="A251" r:id="rId219" tooltip="Lowell, Massachusetts" display="https://en.wikipedia.org/wiki/Lowell,_Massachusetts" xr:uid="{1F945F81-C55B-4F0B-99E8-FBBB177CA02C}"/>
-    <hyperlink ref="A252" r:id="rId220" tooltip="Odessa, Texas" display="https://en.wikipedia.org/wiki/Odessa,_Texas" xr:uid="{610148C5-9861-4345-B74E-AE41B197C3D8}"/>
-    <hyperlink ref="A253" r:id="rId221" tooltip="High Point, North Carolina" display="https://en.wikipedia.org/wiki/High_Point,_North_Carolina" xr:uid="{9FB4C72E-5A47-4100-9E76-E5169ED9B159}"/>
-    <hyperlink ref="A254" r:id="rId222" tooltip="League City, Texas" display="https://en.wikipedia.org/wiki/League_City,_Texas" xr:uid="{F76F3E51-A8E8-47A8-99FF-B2D7E35759E6}"/>
-    <hyperlink ref="A255" r:id="rId223" tooltip="Antioch, California" display="https://en.wikipedia.org/wiki/Antioch,_California" xr:uid="{7C81C2F2-1150-4203-A0CD-960290CFDA84}"/>
-    <hyperlink ref="A256" r:id="rId224" tooltip="Richardson, Texas" display="https://en.wikipedia.org/wiki/Richardson,_Texas" xr:uid="{1EE11818-B344-464A-9CB9-57D1F85D5005}"/>
-    <hyperlink ref="A257" r:id="rId225" tooltip="Goodyear, Arizona" display="https://en.wikipedia.org/wiki/Goodyear,_Arizona" xr:uid="{BAEBEBD8-4ABB-4DD9-8DEB-998A37836DD0}"/>
-    <hyperlink ref="A258" r:id="rId226" tooltip="Pompano Beach, Florida" display="https://en.wikipedia.org/wiki/Pompano_Beach,_Florida" xr:uid="{CD0F4287-8AEE-4919-933A-DA0A384BB6E7}"/>
-    <hyperlink ref="A259" r:id="rId227" tooltip="Nampa, Idaho" display="https://en.wikipedia.org/wiki/Nampa,_Idaho" xr:uid="{550158AD-5E3F-41BB-A100-323D10DF3F8C}"/>
-    <hyperlink ref="A260" r:id="rId228" tooltip="Menifee, California" display="https://en.wikipedia.org/wiki/Menifee,_California" xr:uid="{296E559B-CC29-499E-BEE5-B4BAA9FE48CA}"/>
-    <hyperlink ref="A261" r:id="rId229" tooltip="Las Cruces, New Mexico" display="https://en.wikipedia.org/wiki/Las_Cruces,_New_Mexico" xr:uid="{E71D585B-BAB4-435C-994F-91A64FA21551}"/>
-    <hyperlink ref="A262" r:id="rId230" tooltip="Clearwater, Florida" display="https://en.wikipedia.org/wiki/Clearwater,_Florida" xr:uid="{B958717E-7CA8-43EC-B2B1-7B84B67DB9CF}"/>
-    <hyperlink ref="A263" r:id="rId231" tooltip="West Jordan, Utah" display="https://en.wikipedia.org/wiki/West_Jordan,_Utah" xr:uid="{F31A29F5-E17C-4EED-A6DA-85EA51C6270F}"/>
-    <hyperlink ref="A264" r:id="rId232" tooltip="New Braunfels, Texas" display="https://en.wikipedia.org/wiki/New_Braunfels,_Texas" xr:uid="{36227FAE-FC19-497F-A359-B256B6602824}"/>
-    <hyperlink ref="A265" r:id="rId233" tooltip="Manchester, New Hampshire" display="https://en.wikipedia.org/wiki/Manchester,_New_Hampshire" xr:uid="{18E7ED5D-3617-4BB3-990E-DC38DBBA9C71}"/>
-    <hyperlink ref="A266" r:id="rId234" tooltip="Miami Gardens, Florida" display="https://en.wikipedia.org/wiki/Miami_Gardens,_Florida" xr:uid="{04D4CFA2-AF3B-42F3-95F6-8CD0675767C5}"/>
-    <hyperlink ref="A267" r:id="rId235" tooltip="Waterbury, Connecticut" display="https://en.wikipedia.org/wiki/Waterbury,_Connecticut" xr:uid="{84C7295B-817B-472B-A4C0-C49A297B9A9A}"/>
-    <hyperlink ref="A268" r:id="rId236" tooltip="Provo, Utah" display="https://en.wikipedia.org/wiki/Provo,_Utah" xr:uid="{5AD91705-1191-4C84-AC0B-01D5EC8AC7F2}"/>
-    <hyperlink ref="A269" r:id="rId237" tooltip="Evansville, Indiana" display="https://en.wikipedia.org/wiki/Evansville,_Indiana" xr:uid="{3D93E37A-4A9F-4771-BD72-DDEB60DE23B9}"/>
-    <hyperlink ref="A270" r:id="rId238" tooltip="Richmond, California" display="https://en.wikipedia.org/wiki/Richmond,_California" xr:uid="{BC72BE65-1043-4A1B-A9D8-5DC9A63902E0}"/>
-    <hyperlink ref="A271" r:id="rId239" tooltip="Westminster, Colorado" display="https://en.wikipedia.org/wiki/Westminster,_Colorado" xr:uid="{84D5954E-F995-42A0-B3A3-9181430599C4}"/>
-    <hyperlink ref="A272" r:id="rId240" tooltip="Elgin, Illinois" display="https://en.wikipedia.org/wiki/Elgin,_Illinois" xr:uid="{14C7D917-1DBD-4DBE-AB53-22E21388622F}"/>
-    <hyperlink ref="A273" r:id="rId241" tooltip="Conroe, Texas" display="https://en.wikipedia.org/wiki/Conroe,_Texas" xr:uid="{DD9C3E1A-980B-4666-9F2E-1D4952CCB128}"/>
-    <hyperlink ref="A274" r:id="rId242" tooltip="Greeley, Colorado" display="https://en.wikipedia.org/wiki/Greeley,_Colorado" xr:uid="{8CA4985B-2372-4D79-ACD7-4A4DE06DED0A}"/>
-    <hyperlink ref="A275" r:id="rId243" tooltip="Lansing, Michigan" display="https://en.wikipedia.org/wiki/Lansing,_Michigan" xr:uid="{2116C234-776D-4DB9-B3EB-83DD6B8F3FE3}"/>
-    <hyperlink ref="A276" r:id="rId244" tooltip="Buckeye, Arizona" display="https://en.wikipedia.org/wiki/Buckeye,_Arizona" xr:uid="{E0F4F41E-7A15-4A60-8E2D-5897BF290AFB}"/>
-    <hyperlink ref="A277" r:id="rId245" tooltip="Tuscaloosa, Alabama" display="https://en.wikipedia.org/wiki/Tuscaloosa,_Alabama" xr:uid="{D2EB49D3-2B35-47D9-A542-97AF06897478}"/>
-    <hyperlink ref="A278" r:id="rId246" tooltip="Allen, Texas" display="https://en.wikipedia.org/wiki/Allen,_Texas" xr:uid="{2043AED9-EE1B-4494-A41D-8667FB36610C}"/>
-    <hyperlink ref="A279" r:id="rId247" tooltip="Carlsbad, California" display="https://en.wikipedia.org/wiki/Carlsbad,_California" xr:uid="{23371DB8-7A80-4499-A75C-6DCDDC79CFEC}"/>
-    <hyperlink ref="A280" r:id="rId248" tooltip="Everett, Washington" display="https://en.wikipedia.org/wiki/Everett,_Washington" xr:uid="{128C008B-C6F6-46D6-B970-36D965AB5D36}"/>
-    <hyperlink ref="A281" r:id="rId249" tooltip="Springfield, Illinois" display="https://en.wikipedia.org/wiki/Springfield,_Illinois" xr:uid="{A78A1E63-664D-48E0-98D9-673EE26BB55F}"/>
-    <hyperlink ref="A282" r:id="rId250" tooltip="Beaumont, Texas" display="https://en.wikipedia.org/wiki/Beaumont,_Texas" xr:uid="{853FD3C3-E301-42C8-AF72-298737C51441}"/>
-    <hyperlink ref="A283" r:id="rId251" tooltip="Murrieta, California" display="https://en.wikipedia.org/wiki/Murrieta,_California" xr:uid="{8560D580-1E8B-4E59-9D71-FCFAD494DB60}"/>
-    <hyperlink ref="A284" r:id="rId252" tooltip="Rio Rancho, New Mexico" display="https://en.wikipedia.org/wiki/Rio_Rancho,_New_Mexico" xr:uid="{A1EF8FBB-23F3-4470-BFF8-0C16173BC62A}"/>
-    <hyperlink ref="A285" r:id="rId253" tooltip="Temecula, California" display="https://en.wikipedia.org/wiki/Temecula,_California" xr:uid="{F8C1865E-A75B-4898-A977-1D24561A1D8E}"/>
-    <hyperlink ref="A286" r:id="rId254" tooltip="Concord, North Carolina" display="https://en.wikipedia.org/wiki/Concord,_North_Carolina" xr:uid="{DBEC8C1F-7E06-47E7-9CC0-732522DC5A0C}"/>
-    <hyperlink ref="A287" r:id="rId255" tooltip="Tyler, Texas" display="https://en.wikipedia.org/wiki/Tyler,_Texas" xr:uid="{7F383203-7C39-4212-978E-5A8AE462EDBC}"/>
-    <hyperlink ref="A288" r:id="rId256" tooltip="Davie, Florida" display="https://en.wikipedia.org/wiki/Davie,_Florida" xr:uid="{20723A51-8C85-444B-A75B-6638141CE779}"/>
-    <hyperlink ref="A289" r:id="rId257" tooltip="South Fulton, Georgia" display="https://en.wikipedia.org/wiki/South_Fulton,_Georgia" xr:uid="{73C75744-21C3-4146-B697-8210E551B66C}"/>
-    <hyperlink ref="A290" r:id="rId258" tooltip="Peoria, Illinois" display="https://en.wikipedia.org/wiki/Peoria,_Illinois" xr:uid="{8E3D2518-DAA1-49C2-8776-E02E6545B601}"/>
-    <hyperlink ref="A291" r:id="rId259" tooltip="Sparks, Nevada" display="https://en.wikipedia.org/wiki/Sparks,_Nevada" xr:uid="{6A4552ED-252D-4AB0-9EBE-8CC2E3115E5A}"/>
-    <hyperlink ref="A292" r:id="rId260" tooltip="Gresham, Oregon" display="https://en.wikipedia.org/wiki/Gresham,_Oregon" xr:uid="{ECC64D24-C00A-4C6B-B978-C093D8324F20}"/>
-    <hyperlink ref="A293" r:id="rId261" tooltip="Santa Maria, California" display="https://en.wikipedia.org/wiki/Santa_Maria,_California" xr:uid="{A888E5F6-EA84-4F58-A3B5-B0D41858EDFB}"/>
-    <hyperlink ref="A294" r:id="rId262" tooltip="Pueblo, Colorado" display="https://en.wikipedia.org/wiki/Pueblo,_Colorado" xr:uid="{2998C889-8570-45C1-9623-16B2D5FC4D32}"/>
-    <hyperlink ref="A295" r:id="rId263" tooltip="Hillsboro, Oregon" display="https://en.wikipedia.org/wiki/Hillsboro,_Oregon" xr:uid="{8327BC54-94CC-49B0-8051-C52DAB9F7A86}"/>
-    <hyperlink ref="A297" r:id="rId264" tooltip="Sugar Land, Texas" display="https://en.wikipedia.org/wiki/Sugar_Land,_Texas" xr:uid="{29F7F70C-FA86-4466-967B-A243148BA870}"/>
-    <hyperlink ref="A299" r:id="rId265" tooltip="Downey, California" display="https://en.wikipedia.org/wiki/Downey,_California" xr:uid="{B743D911-1E08-4AAC-8A82-105F6B0F1BD1}"/>
-    <hyperlink ref="A300" r:id="rId266" tooltip="Costa Mesa, California" display="https://en.wikipedia.org/wiki/Costa_Mesa,_California" xr:uid="{7A6973C9-C4E6-473B-BC32-E19FE8FF438C}"/>
-    <hyperlink ref="A301" r:id="rId267" tooltip="Centennial, Colorado" display="https://en.wikipedia.org/wiki/Centennial,_Colorado" xr:uid="{6327416D-84D1-47C4-B190-BF3E2A59BA2D}"/>
-    <hyperlink ref="A302" r:id="rId268" tooltip="Edinburg, Texas" display="https://en.wikipedia.org/wiki/Edinburg,_Texas" xr:uid="{2C9AFD68-19D2-4C61-8A4C-A20B6045ABB7}"/>
-    <hyperlink ref="A303" r:id="rId269" tooltip="Spokane Valley, Washington" display="https://en.wikipedia.org/wiki/Spokane_Valley,_Washington" xr:uid="{020B1BBE-B3DE-435B-83FD-DF7CED5056E8}"/>
-    <hyperlink ref="A304" r:id="rId270" tooltip="Jurupa Valley, California" display="https://en.wikipedia.org/wiki/Jurupa_Valley,_California" xr:uid="{295EA295-3E75-4397-AAFC-A719EF4437E8}"/>
-    <hyperlink ref="A305" r:id="rId271" tooltip="Bend, Oregon" display="https://en.wikipedia.org/wiki/Bend,_Oregon" xr:uid="{7E1F6E81-20AC-4E82-ADB7-017D2574DFD3}"/>
-    <hyperlink ref="A306" r:id="rId272" tooltip="West Covina, California" display="https://en.wikipedia.org/wiki/West_Covina,_California" xr:uid="{69575739-061B-4DA9-8FFC-159E9B3DA164}"/>
-    <hyperlink ref="A307" r:id="rId273" tooltip="Boulder, Colorado" display="https://en.wikipedia.org/wiki/Boulder,_Colorado" xr:uid="{48EB3296-B8FB-46E8-8D40-D1E2B21391D6}"/>
-    <hyperlink ref="A308" r:id="rId274" tooltip="Palm Coast, Florida" display="https://en.wikipedia.org/wiki/Palm_Coast,_Florida" xr:uid="{0DEF77AF-5FEB-4BB3-9800-CF76C6CB3653}"/>
-    <hyperlink ref="A309" r:id="rId275" tooltip="Lee's Summit, Missouri" display="https://en.wikipedia.org/wiki/Lee%27s_Summit,_Missouri" xr:uid="{CD41760B-D163-41AE-8194-32ED07FC2AB3}"/>
-    <hyperlink ref="A310" r:id="rId276" tooltip="Dearborn, Michigan" display="https://en.wikipedia.org/wiki/Dearborn,_Michigan" xr:uid="{E84116F0-6AE8-42B0-9503-2BF0ACE98582}"/>
-    <hyperlink ref="A311" r:id="rId277" tooltip="Green Bay, Wisconsin" display="https://en.wikipedia.org/wiki/Green_Bay,_Wisconsin" xr:uid="{BC32108E-8CCC-4531-A1AB-E0EFF02FC0DB}"/>
-    <hyperlink ref="A312" r:id="rId278" tooltip="St. George, Utah" display="https://en.wikipedia.org/wiki/St._George,_Utah" xr:uid="{0EF65130-5D66-4725-9CD9-9D5AEE02C313}"/>
-    <hyperlink ref="A314" r:id="rId279" tooltip="Brockton, Massachusetts" display="https://en.wikipedia.org/wiki/Brockton,_Massachusetts" xr:uid="{EE39A630-758B-4FAB-807D-AFF78DE08337}"/>
-    <hyperlink ref="A315" r:id="rId280" tooltip="Renton, Washington" display="https://en.wikipedia.org/wiki/Renton,_Washington" xr:uid="{00691DBE-1C7A-4929-8D13-7B896257CB2A}"/>
-    <hyperlink ref="A316" r:id="rId281" tooltip="Sandy Springs, Georgia" display="https://en.wikipedia.org/wiki/Sandy_Springs,_Georgia" xr:uid="{4EFA647B-2F55-44E4-8209-FC1F4AF9324B}"/>
-    <hyperlink ref="A317" r:id="rId282" tooltip="Rialto, California" display="https://en.wikipedia.org/wiki/Rialto,_California" xr:uid="{E501ED92-6B0C-4BE9-A742-5DE3A6B31C8F}"/>
-    <hyperlink ref="A318" r:id="rId283" tooltip="El Monte, California" display="https://en.wikipedia.org/wiki/El_Monte,_California" xr:uid="{ECB59E81-4A97-453D-8324-F9A4E42A8654}"/>
-    <hyperlink ref="A319" r:id="rId284" tooltip="Vacaville, California" display="https://en.wikipedia.org/wiki/Vacaville,_California" xr:uid="{44279042-4D9B-4080-AE32-A98C4C48B7A8}"/>
-    <hyperlink ref="A320" r:id="rId285" tooltip="Fishers, Indiana" display="https://en.wikipedia.org/wiki/Fishers,_Indiana" xr:uid="{402E2B4B-044E-41DF-915D-AB38ECD8AD70}"/>
-    <hyperlink ref="A321" r:id="rId286" tooltip="South Bend, Indiana" display="https://en.wikipedia.org/wiki/South_Bend,_Indiana" xr:uid="{73A00911-2D47-4E8A-A351-B4772D595DFE}"/>
-    <hyperlink ref="A322" r:id="rId287" tooltip="Carmel, Indiana" display="https://en.wikipedia.org/wiki/Carmel,_Indiana" xr:uid="{09A6F8BE-B0DF-4B38-820B-4B8794A44A5A}"/>
-    <hyperlink ref="A323" r:id="rId288" tooltip="Yuma, Arizona" display="https://en.wikipedia.org/wiki/Yuma,_Arizona" xr:uid="{39FF4BB3-6EEB-456E-BE88-EA97A18376E7}"/>
-    <hyperlink ref="A324" r:id="rId289" tooltip="Burbank, California" display="https://en.wikipedia.org/wiki/Burbank,_California" xr:uid="{6804245F-5620-40F0-8E47-04417D9DA751}"/>
-    <hyperlink ref="A325" r:id="rId290" tooltip="Lynn, Massachusetts" display="https://en.wikipedia.org/wiki/Lynn,_Massachusetts" xr:uid="{0737B5F0-2E3B-4CBF-9406-0EE9A67EF2B5}"/>
-    <hyperlink ref="A326" r:id="rId291" tooltip="Quincy, Massachusetts" display="https://en.wikipedia.org/wiki/Quincy,_Massachusetts" xr:uid="{8B0AAB2B-AA5C-4E2C-BA62-B9C8BAAF5207}"/>
-    <hyperlink ref="A327" r:id="rId292" tooltip="El Cajon, California" display="https://en.wikipedia.org/wiki/El_Cajon,_California" xr:uid="{9EDD555C-B7F6-40C9-B7E2-3B50F65F4560}"/>
-    <hyperlink ref="A328" r:id="rId293" tooltip="Fayetteville, Arkansas" display="https://en.wikipedia.org/wiki/Fayetteville,_Arkansas" xr:uid="{2E5FC15A-AF54-4BF7-9AA5-69AF819F062D}"/>
-    <hyperlink ref="A330" r:id="rId294" tooltip="San Mateo, California" display="https://en.wikipedia.org/wiki/San_Mateo,_California" xr:uid="{A4DEEBC7-483A-48D5-9277-289D8F450BDB}"/>
-    <hyperlink ref="A331" r:id="rId295" tooltip="Chico, California" display="https://en.wikipedia.org/wiki/Chico,_California" xr:uid="{CD6EB241-A61E-4451-A74A-CA5412254C62}"/>
-    <hyperlink ref="A332" r:id="rId296" tooltip="Inglewood, California" display="https://en.wikipedia.org/wiki/Inglewood,_California" xr:uid="{88256F8E-1302-4138-BFEA-37C5A32B5E51}"/>
-    <hyperlink ref="A333" r:id="rId297" tooltip="Wichita Falls, Texas" display="https://en.wikipedia.org/wiki/Wichita_Falls,_Texas" xr:uid="{6F93A719-EED6-4A9C-B438-4DE9D8E12E70}"/>
-    <hyperlink ref="A334" r:id="rId298" tooltip="Boca Raton, Florida" display="https://en.wikipedia.org/wiki/Boca_Raton,_Florida" xr:uid="{40086BB0-4537-4537-8A7F-AD1DB13E49F1}"/>
-    <hyperlink ref="A335" r:id="rId299" tooltip="Hesperia, California" display="https://en.wikipedia.org/wiki/Hesperia,_California" xr:uid="{5A282B4D-DB62-4EDE-9251-B12B80A02CF6}"/>
-    <hyperlink ref="A336" r:id="rId300" tooltip="Daly City, California" display="https://en.wikipedia.org/wiki/Daly_City,_California" xr:uid="{273F395E-8A2C-4A59-B9C0-6BBAF95CE82C}"/>
-    <hyperlink ref="A338" r:id="rId301" tooltip="Georgetown, Texas" display="https://en.wikipedia.org/wiki/Georgetown,_Texas" xr:uid="{F6B17462-7C74-498E-B740-65A4E7749CE7}"/>
-    <hyperlink ref="A339" r:id="rId302" tooltip="New Bedford, Massachusetts" display="https://en.wikipedia.org/wiki/New_Bedford,_Massachusetts" xr:uid="{25990844-1D54-45CB-A483-30DD8FBB0CD2}"/>
-    <hyperlink ref="A340" r:id="rId303" tooltip="Albany, New York" display="https://en.wikipedia.org/wiki/Albany,_New_York" xr:uid="{134E9866-C107-4A21-AECB-C63388B25232}"/>
-    <hyperlink ref="A341" r:id="rId304" tooltip="Davenport, Iowa" display="https://en.wikipedia.org/wiki/Davenport,_Iowa" xr:uid="{ABF3CE13-C477-4AD0-92A4-19A33CE8505D}"/>
-    <hyperlink ref="A342" r:id="rId305" tooltip="Plantation, Florida" display="https://en.wikipedia.org/wiki/Plantation,_Florida" xr:uid="{F9A40EA9-2F97-41AC-9CB0-6C87E2448DA0}"/>
-    <hyperlink ref="A343" r:id="rId306" tooltip="Deltona, Florida" display="https://en.wikipedia.org/wiki/Deltona,_Florida" xr:uid="{F86B9F1E-0353-40B1-87DA-D74935E2F1E2}"/>
-    <hyperlink ref="A344" r:id="rId307" tooltip="Federal Way, Washington" display="https://en.wikipedia.org/wiki/Federal_Way,_Washington" xr:uid="{6A733CDF-C6F6-4A3F-86ED-0B1C45801AEA}"/>
-    <hyperlink ref="A345" r:id="rId308" tooltip="San Angelo, Texas" display="https://en.wikipedia.org/wiki/San_Angelo,_Texas" xr:uid="{BF3DB560-73FF-4047-A1A3-D9F70CDFC2F0}"/>
-    <hyperlink ref="A346" r:id="rId309" tooltip="Tracy, California" display="https://en.wikipedia.org/wiki/Tracy,_California" xr:uid="{690292EE-71CB-4C84-8011-880C6516847C}"/>
-    <hyperlink ref="A347" r:id="rId310" tooltip="Sunrise, Florida" display="https://en.wikipedia.org/wiki/Sunrise,_Florida" xr:uid="{D6743DD7-E0E4-4D89-9538-92361E1ED4C2}"/>
+    <hyperlink ref="A126" r:id="rId103" tooltip="Mobile, Alabama" display="https://en.wikipedia.org/wiki/Mobile,_Alabama" xr:uid="{4E2896C7-D20A-4C4D-80BA-6FA7EE84347E}"/>
+    <hyperlink ref="A127" r:id="rId104" tooltip="Oxnard, California" display="https://en.wikipedia.org/wiki/Oxnard,_California" xr:uid="{052FB3E4-9739-4330-B5B5-9CD746CCCA7E}"/>
+    <hyperlink ref="A128" r:id="rId105" tooltip="Grand Rapids, Michigan" display="https://en.wikipedia.org/wiki/Grand_Rapids,_Michigan" xr:uid="{8D0C128B-FFDC-481C-A82A-2478374C7FFC}"/>
+    <hyperlink ref="A129" r:id="rId106" tooltip="Peoria, Arizona" display="https://en.wikipedia.org/wiki/Peoria,_Arizona" xr:uid="{42DE2250-B81C-4119-B875-3B3D2BBC0774}"/>
+    <hyperlink ref="A130" r:id="rId107" tooltip="Vancouver, Washington" display="https://en.wikipedia.org/wiki/Vancouver,_Washington" xr:uid="{56DB179A-8427-415C-820F-20758DEF26F4}"/>
+    <hyperlink ref="A131" r:id="rId108" tooltip="Knoxville, Tennessee" display="https://en.wikipedia.org/wiki/Knoxville,_Tennessee" xr:uid="{3191FCC6-6BD4-4A6D-AC10-B7329A152ABD}"/>
+    <hyperlink ref="A132" r:id="rId109" tooltip="Birmingham, Alabama" display="https://en.wikipedia.org/wiki/Birmingham,_Alabama" xr:uid="{B0F1434B-2180-4728-BBB7-DC5D157943C1}"/>
+    <hyperlink ref="A133" r:id="rId110" tooltip="Montgomery, Alabama" display="https://en.wikipedia.org/wiki/Montgomery,_Alabama" xr:uid="{243C3328-7F74-4607-A5BF-0DB07F7695E3}"/>
+    <hyperlink ref="A134" r:id="rId111" tooltip="Providence, Rhode Island" display="https://en.wikipedia.org/wiki/Providence,_Rhode_Island" xr:uid="{B18F437D-0BD6-49A0-B395-48E8ACF5A67A}"/>
+    <hyperlink ref="A135" r:id="rId112" tooltip="Huntington Beach, California" display="https://en.wikipedia.org/wiki/Huntington_Beach,_California" xr:uid="{EC38142B-2562-4B33-A90A-23AA220C0C86}"/>
+    <hyperlink ref="A136" r:id="rId113" tooltip="Brownsville, Texas" display="https://en.wikipedia.org/wiki/Brownsville,_Texas" xr:uid="{C7CAF846-2A11-42FE-8CCC-19177CAE3C57}"/>
+    <hyperlink ref="A137" r:id="rId114" tooltip="Chattanooga, Tennessee" display="https://en.wikipedia.org/wiki/Chattanooga,_Tennessee" xr:uid="{7DD8093A-1E37-4F1C-96D2-248C52349C1E}"/>
+    <hyperlink ref="A138" r:id="rId115" tooltip="Fort Lauderdale, Florida" display="https://en.wikipedia.org/wiki/Fort_Lauderdale,_Florida" xr:uid="{228D6E06-E1E1-40D8-8D34-B05A4AF7959C}"/>
+    <hyperlink ref="A139" r:id="rId116" tooltip="Tempe, Arizona" display="https://en.wikipedia.org/wiki/Tempe,_Arizona" xr:uid="{9A6B5A9C-D0F6-446D-9C4E-67078BB98A2E}"/>
+    <hyperlink ref="A140" r:id="rId117" tooltip="Akron, Ohio" display="https://en.wikipedia.org/wiki/Akron,_Ohio" xr:uid="{819F738E-195E-463F-AB6B-389E157E76F2}"/>
+    <hyperlink ref="A141" r:id="rId118" tooltip="Clarksville, Tennessee" display="https://en.wikipedia.org/wiki/Clarksville,_Tennessee" xr:uid="{60A80EAF-F3C7-408C-A885-091C7F98C21C}"/>
+    <hyperlink ref="A142" r:id="rId119" tooltip="Ontario, California" display="https://en.wikipedia.org/wiki/Ontario,_California" xr:uid="{5ADAA54E-67DF-4A47-A555-F8A040679E6E}"/>
+    <hyperlink ref="A144" r:id="rId120" tooltip="Elk Grove, California" display="https://en.wikipedia.org/wiki/Elk_Grove,_California" xr:uid="{7D8A5CB7-CE45-47B5-9BA9-EC23CD3121FC}"/>
+    <hyperlink ref="A145" r:id="rId121" tooltip="Cary, North Carolina" display="https://en.wikipedia.org/wiki/Cary,_North_Carolina" xr:uid="{79238080-FBEB-413C-B4EC-25113F093DAB}"/>
+    <hyperlink ref="A146" r:id="rId122" tooltip="Salem, Oregon" display="https://en.wikipedia.org/wiki/Salem,_Oregon" xr:uid="{57C4AD57-3BE4-4858-B3CE-4383A20849AE}"/>
+    <hyperlink ref="A147" r:id="rId123" tooltip="Pembroke Pines, Florida" display="https://en.wikipedia.org/wiki/Pembroke_Pines,_Florida" xr:uid="{5504AF73-E1C8-496D-9493-736EDFDEB61C}"/>
+    <hyperlink ref="A148" r:id="rId124" tooltip="Eugene, Oregon" display="https://en.wikipedia.org/wiki/Eugene,_Oregon" xr:uid="{3CC9226D-8DBF-4F8F-A94B-21C0F2968F0D}"/>
+    <hyperlink ref="A149" r:id="rId125" tooltip="Santa Rosa, California" display="https://en.wikipedia.org/wiki/Santa_Rosa,_California" xr:uid="{A9BBF8A8-C94B-4BA8-A909-D6DAB891141D}"/>
+    <hyperlink ref="A150" r:id="rId126" tooltip="Rancho Cucamonga, California" display="https://en.wikipedia.org/wiki/Rancho_Cucamonga,_California" xr:uid="{920CC947-E031-4EB0-986D-9A97014345D7}"/>
+    <hyperlink ref="A151" r:id="rId127" tooltip="Shreveport, Louisiana" display="https://en.wikipedia.org/wiki/Shreveport,_Louisiana" xr:uid="{C4A0CDD8-B0FF-4BDA-981D-6A3CE676142A}"/>
+    <hyperlink ref="A152" r:id="rId128" tooltip="Garden Grove, California" display="https://en.wikipedia.org/wiki/Garden_Grove,_California" xr:uid="{A54A8506-CC2D-4453-9241-07C4C35486A9}"/>
+    <hyperlink ref="A153" r:id="rId129" tooltip="Oceanside, California" display="https://en.wikipedia.org/wiki/Oceanside,_California" xr:uid="{B5E0D532-AA0F-4F4A-B48A-DDB52F59614B}"/>
+    <hyperlink ref="A154" r:id="rId130" tooltip="Fort Collins, Colorado" display="https://en.wikipedia.org/wiki/Fort_Collins,_Colorado" xr:uid="{48526A50-3DE3-4820-B7FC-1F8EA26E1FF1}"/>
+    <hyperlink ref="A155" r:id="rId131" tooltip="Springfield, Missouri" display="https://en.wikipedia.org/wiki/Springfield,_Missouri" xr:uid="{159962FC-4A24-49B3-939A-BF554AD8F9CE}"/>
+    <hyperlink ref="A156" r:id="rId132" tooltip="Murfreesboro, Tennessee" display="https://en.wikipedia.org/wiki/Murfreesboro,_Tennessee" xr:uid="{028986A8-13D8-45DB-8308-38F5D6975394}"/>
+    <hyperlink ref="A157" r:id="rId133" tooltip="Surprise, Arizona" display="https://en.wikipedia.org/wiki/Surprise,_Arizona" xr:uid="{9F81C077-8E62-4CE0-B2F1-3D8ED9546E89}"/>
+    <hyperlink ref="A158" r:id="rId134" tooltip="Lancaster, California" display="https://en.wikipedia.org/wiki/Lancaster,_California" xr:uid="{BA04C0C3-2052-4003-A556-BE985789E293}"/>
+    <hyperlink ref="A159" r:id="rId135" tooltip="Denton, Texas" display="https://en.wikipedia.org/wiki/Denton,_Texas" xr:uid="{C4DEA4D8-6231-44D9-BE26-5A855CCEE36D}"/>
+    <hyperlink ref="A160" r:id="rId136" tooltip="Roseville, California" display="https://en.wikipedia.org/wiki/Roseville,_California" xr:uid="{AB952918-E34D-40D6-8C85-3CC456F7EEE4}"/>
+    <hyperlink ref="A161" r:id="rId137" tooltip="Palmdale, California" display="https://en.wikipedia.org/wiki/Palmdale,_California" xr:uid="{5D4C2C43-9935-4AF9-A0A2-B3546E301F66}"/>
+    <hyperlink ref="A162" r:id="rId138" tooltip="Corona, California" display="https://en.wikipedia.org/wiki/Corona,_California" xr:uid="{79F07F89-247B-4564-B1CF-63DA0443AD2D}"/>
+    <hyperlink ref="A163" r:id="rId139" tooltip="Salinas, California" display="https://en.wikipedia.org/wiki/Salinas,_California" xr:uid="{0A5A2FD9-D666-4D98-8976-B306D0B0C5E2}"/>
+    <hyperlink ref="A164" r:id="rId140" tooltip="Killeen, Texas" display="https://en.wikipedia.org/wiki/Killeen,_Texas" xr:uid="{9DF4AF29-351F-4CA2-9882-62B0E04705C0}"/>
+    <hyperlink ref="A165" r:id="rId141" tooltip="Paterson, New Jersey" display="https://en.wikipedia.org/wiki/Paterson,_New_Jersey" xr:uid="{030A6D78-319E-4361-81DF-9FA91B5F8363}"/>
+    <hyperlink ref="A167" r:id="rId142" tooltip="Hollywood, Florida" display="https://en.wikipedia.org/wiki/Hollywood,_Florida" xr:uid="{2E514F97-08AE-4C83-8AA5-249046DF2182}"/>
+    <hyperlink ref="A168" r:id="rId143" tooltip="Hayward, California" display="https://en.wikipedia.org/wiki/Hayward,_California" xr:uid="{758E4979-EA25-41AD-9A83-DAE7CABC51CB}"/>
+    <hyperlink ref="A169" r:id="rId144" tooltip="Charleston, South Carolina" display="https://en.wikipedia.org/wiki/Charleston,_South_Carolina" xr:uid="{ABF30A89-881F-4D1E-A027-BD2DF9FA7396}"/>
+    <hyperlink ref="A171" r:id="rId145" tooltip="Lakewood, Colorado" display="https://en.wikipedia.org/wiki/Lakewood,_Colorado" xr:uid="{D4B8E640-228C-40FA-A462-8570AB31B310}"/>
+    <hyperlink ref="A172" r:id="rId146" tooltip="Sunnyvale, California" display="https://en.wikipedia.org/wiki/Sunnyvale,_California" xr:uid="{868F929C-5F4D-4AA9-9644-AA6FAFE84F3F}"/>
+    <hyperlink ref="A173" r:id="rId147" tooltip="Bellevue, Washington" display="https://en.wikipedia.org/wiki/Bellevue,_Washington" xr:uid="{6F9C2962-8946-46D9-A375-62E5C91270D7}"/>
+    <hyperlink ref="A174" r:id="rId148" tooltip="Naperville, Illinois" display="https://en.wikipedia.org/wiki/Naperville,_Illinois" xr:uid="{4DB54CD8-BD51-4D4C-9FD1-30ECAFA73408}"/>
+    <hyperlink ref="A175" r:id="rId149" tooltip="Joliet, Illinois" display="https://en.wikipedia.org/wiki/Joliet,_Illinois" xr:uid="{2B68DF39-77FA-4587-91BC-440C7E1FAEA9}"/>
+    <hyperlink ref="A176" r:id="rId150" tooltip="Bridgeport, Connecticut" display="https://en.wikipedia.org/wiki/Bridgeport,_Connecticut" xr:uid="{6C639E49-E2CF-43E5-A98A-E0DB9579406B}"/>
+    <hyperlink ref="A177" r:id="rId151" tooltip="Mesquite, Texas" display="https://en.wikipedia.org/wiki/Mesquite,_Texas" xr:uid="{95F60B5B-76CA-456E-8F1E-9C9BBDB8D150}"/>
+    <hyperlink ref="A178" r:id="rId152" tooltip="Pasadena, Texas" display="https://en.wikipedia.org/wiki/Pasadena,_Texas" xr:uid="{59E07B82-9CBF-494B-9C62-E014257ECB57}"/>
+    <hyperlink ref="A179" r:id="rId153" tooltip="Olathe, Kansas" display="https://en.wikipedia.org/wiki/Olathe,_Kansas" xr:uid="{8A551723-EC13-4EAC-A759-3831FCDE0FBA}"/>
+    <hyperlink ref="A180" r:id="rId154" tooltip="Escondido, California" display="https://en.wikipedia.org/wiki/Escondido,_California" xr:uid="{7C50450E-C974-44E4-B1DD-C67F306B77D9}"/>
+    <hyperlink ref="A181" r:id="rId155" tooltip="Savannah, Georgia" display="https://en.wikipedia.org/wiki/Savannah,_Georgia" xr:uid="{B437D653-1143-4A10-BADC-D286B6ACC723}"/>
+    <hyperlink ref="A182" r:id="rId156" tooltip="McAllen, Texas" display="https://en.wikipedia.org/wiki/McAllen,_Texas" xr:uid="{AEC35262-3478-445B-84D6-751CD4AB3EB8}"/>
+    <hyperlink ref="A183" r:id="rId157" tooltip="Gainesville, Florida" display="https://en.wikipedia.org/wiki/Gainesville,_Florida" xr:uid="{515430DE-7083-474C-B331-11441A93126F}"/>
+    <hyperlink ref="A184" r:id="rId158" tooltip="Pomona, California" display="https://en.wikipedia.org/wiki/Pomona,_California" xr:uid="{B1094DCC-91EE-4D42-93BC-775D727B4BFB}"/>
+    <hyperlink ref="A185" r:id="rId159" tooltip="Rockford, Illinois" display="https://en.wikipedia.org/wiki/Rockford,_Illinois" xr:uid="{6D481027-4AFF-44F2-88E1-76967CC0E2A6}"/>
+    <hyperlink ref="A186" r:id="rId160" tooltip="Thornton, Colorado" display="https://en.wikipedia.org/wiki/Thornton,_Colorado" xr:uid="{089AD7E4-304F-45D7-8568-F69C04962229}"/>
+    <hyperlink ref="A187" r:id="rId161" tooltip="Waco, Texas" display="https://en.wikipedia.org/wiki/Waco,_Texas" xr:uid="{E2E37336-2BFF-4BA9-B2E9-2AB8AA0B9AA8}"/>
+    <hyperlink ref="A188" r:id="rId162" tooltip="Visalia, California" display="https://en.wikipedia.org/wiki/Visalia,_California" xr:uid="{29E9B44C-BD44-4415-8353-32105E42888C}"/>
+    <hyperlink ref="A189" r:id="rId163" tooltip="Syracuse, New York" display="https://en.wikipedia.org/wiki/Syracuse,_New_York" xr:uid="{A14C8F93-A81F-4C3D-88E4-2AFE1705D539}"/>
+    <hyperlink ref="A190" r:id="rId164" tooltip="Columbia, South Carolina" display="https://en.wikipedia.org/wiki/Columbia,_South_Carolina" xr:uid="{F4F498F5-0B13-4FF8-A95C-1AA4467DE7C6}"/>
+    <hyperlink ref="A191" r:id="rId165" tooltip="Midland, Texas" display="https://en.wikipedia.org/wiki/Midland,_Texas" xr:uid="{E582A898-E936-4550-A605-650D12038D6D}"/>
+    <hyperlink ref="A192" r:id="rId166" tooltip="Miramar, Florida" display="https://en.wikipedia.org/wiki/Miramar,_Florida" xr:uid="{3BA09F94-2888-4164-BE2A-0AF6F7D7563B}"/>
+    <hyperlink ref="A193" r:id="rId167" tooltip="Palm Bay, Florida" display="https://en.wikipedia.org/wiki/Palm_Bay,_Florida" xr:uid="{7AB8CBCA-ACE3-4F96-97A6-330084EF6E97}"/>
+    <hyperlink ref="A194" r:id="rId168" tooltip="Jackson, Mississippi" display="https://en.wikipedia.org/wiki/Jackson,_Mississippi" xr:uid="{452C5DBB-23EC-47E7-8022-C74105F4066E}"/>
+    <hyperlink ref="A195" r:id="rId169" tooltip="Coral Springs, Florida" display="https://en.wikipedia.org/wiki/Coral_Springs,_Florida" xr:uid="{1E574227-B848-43C2-B9F4-22D0F218B4C4}"/>
+    <hyperlink ref="A196" r:id="rId170" tooltip="Victorville, California" display="https://en.wikipedia.org/wiki/Victorville,_California" xr:uid="{52E5C233-3B9B-4865-A502-6B8E7389212C}"/>
+    <hyperlink ref="A197" r:id="rId171" tooltip="Elizabeth, New Jersey" display="https://en.wikipedia.org/wiki/Elizabeth,_New_Jersey" xr:uid="{C8F9B792-D568-48D5-8A78-2D781C24AF74}"/>
+    <hyperlink ref="A198" r:id="rId172" tooltip="Fullerton, California" display="https://en.wikipedia.org/wiki/Fullerton,_California" xr:uid="{5CBFCC65-14FB-4A2B-8F31-F6946EB55A5C}"/>
+    <hyperlink ref="A199" r:id="rId173" tooltip="Meridian, Idaho" display="https://en.wikipedia.org/wiki/Meridian,_Idaho" xr:uid="{597815BB-8ED0-4939-BF0A-55F4A5E8BC50}"/>
+    <hyperlink ref="A200" r:id="rId174" tooltip="Torrance, California" display="https://en.wikipedia.org/wiki/Torrance,_California" xr:uid="{FF8E2C05-3A0A-4C12-A1C2-C8DDF230745D}"/>
+    <hyperlink ref="A201" r:id="rId175" tooltip="Stamford, Connecticut" display="https://en.wikipedia.org/wiki/Stamford,_Connecticut" xr:uid="{03D2E1BE-0681-44F9-BDC4-01AC870E7E56}"/>
+    <hyperlink ref="A202" r:id="rId176" tooltip="West Valley City, Utah" display="https://en.wikipedia.org/wiki/West_Valley_City,_Utah" xr:uid="{13121615-27BF-4675-A1A6-EAD51C7BD23C}"/>
+    <hyperlink ref="A203" r:id="rId177" tooltip="Orange, California" display="https://en.wikipedia.org/wiki/Orange,_California" xr:uid="{4E6A91BB-9161-49ED-B5BE-6E6167F3E176}"/>
+    <hyperlink ref="A204" r:id="rId178" tooltip="Cedar Rapids, Iowa" display="https://en.wikipedia.org/wiki/Cedar_Rapids,_Iowa" xr:uid="{FEA38046-A2F4-4386-B26C-19A067C94BC4}"/>
+    <hyperlink ref="A205" r:id="rId179" tooltip="Warren, Michigan" display="https://en.wikipedia.org/wiki/Warren,_Michigan" xr:uid="{50A9F933-1332-4090-83DE-72B53CE9FAA0}"/>
+    <hyperlink ref="A207" r:id="rId180" tooltip="New Haven, Connecticut" display="https://en.wikipedia.org/wiki/New_Haven,_Connecticut" xr:uid="{36736AE9-BC59-4B0E-9277-4D6FBE835464}"/>
+    <hyperlink ref="A208" r:id="rId181" tooltip="Kent, Washington" display="https://en.wikipedia.org/wiki/Kent,_Washington" xr:uid="{D5AFC1CD-5101-45C9-AAE5-F44865689E1B}"/>
+    <hyperlink ref="A209" r:id="rId182" tooltip="Dayton, Ohio" display="https://en.wikipedia.org/wiki/Dayton,_Ohio" xr:uid="{31F02388-BE9C-4CE9-97DC-EB6DA4199D2A}"/>
+    <hyperlink ref="A210" r:id="rId183" tooltip="Fargo, North Dakota" display="https://en.wikipedia.org/wiki/Fargo,_North_Dakota" xr:uid="{5386272E-280B-4D18-BA96-A85462C4CCC5}"/>
+    <hyperlink ref="A211" r:id="rId184" tooltip="Lewisville, Texas" display="https://en.wikipedia.org/wiki/Lewisville,_Texas" xr:uid="{7C126BE8-F9E1-4A95-A740-3E8BA349158C}"/>
+    <hyperlink ref="A212" r:id="rId185" tooltip="Carrollton, Texas" display="https://en.wikipedia.org/wiki/Carrollton,_Texas" xr:uid="{D3E15712-3D89-45D0-8D02-1E2E8A00C100}"/>
+    <hyperlink ref="A213" r:id="rId186" tooltip="Round Rock, Texas" display="https://en.wikipedia.org/wiki/Round_Rock,_Texas" xr:uid="{38E0BC55-C7D0-40C4-ACE0-DC353CAEC1E3}"/>
+    <hyperlink ref="A214" r:id="rId187" tooltip="Sterling Heights, Michigan" display="https://en.wikipedia.org/wiki/Sterling_Heights,_Michigan" xr:uid="{17296518-C7F4-4A39-A607-C824D9035787}"/>
+    <hyperlink ref="A215" r:id="rId188" tooltip="Santa Clara, California" display="https://en.wikipedia.org/wiki/Santa_Clara,_California" xr:uid="{0D94D9D7-10A1-4806-80E2-ACF89B9B6747}"/>
+    <hyperlink ref="A216" r:id="rId189" tooltip="Norman, Oklahoma" display="https://en.wikipedia.org/wiki/Norman,_Oklahoma" xr:uid="{C6B26389-B925-4CB9-AA91-0E298A1FADDD}"/>
+    <hyperlink ref="A217" r:id="rId190" tooltip="Abilene, Texas" display="https://en.wikipedia.org/wiki/Abilene,_Texas" xr:uid="{E7C4729C-2C7E-43E8-A6AD-FCC3664ED9A4}"/>
+    <hyperlink ref="A218" r:id="rId191" tooltip="Pearland, Texas" display="https://en.wikipedia.org/wiki/Pearland,_Texas" xr:uid="{9DC3AF36-1C01-4B23-A2FA-5104C8021675}"/>
+    <hyperlink ref="A220" r:id="rId192" tooltip="College Station, Texas" display="https://en.wikipedia.org/wiki/College_Station,_Texas" xr:uid="{D8B084A5-B93D-47A7-8C98-4665850B0F18}"/>
+    <hyperlink ref="A221" r:id="rId193" tooltip="Clovis, California" display="https://en.wikipedia.org/wiki/Clovis,_California" xr:uid="{A5744F83-7207-461E-AAEC-2800B018D389}"/>
+    <hyperlink ref="A222" r:id="rId194" tooltip="West Palm Beach, Florida" display="https://en.wikipedia.org/wiki/West_Palm_Beach,_Florida" xr:uid="{7E4D65CA-0099-4770-8A50-4F4084FAB89E}"/>
+    <hyperlink ref="A223" r:id="rId195" tooltip="Allentown, Pennsylvania" display="https://en.wikipedia.org/wiki/Allentown,_Pennsylvania" xr:uid="{393395BF-6D30-4ED7-BCEE-D1A0798D0761}"/>
+    <hyperlink ref="A224" r:id="rId196" tooltip="North Charleston, South Carolina" display="https://en.wikipedia.org/wiki/North_Charleston,_South_Carolina" xr:uid="{584C8E92-DCE9-4485-B244-A631B2CC3A9C}"/>
+    <hyperlink ref="A225" r:id="rId197" tooltip="Simi Valley, California" display="https://en.wikipedia.org/wiki/Simi_Valley,_California" xr:uid="{829C49A5-275F-478F-AE5B-4EAB3642A1D6}"/>
+    <hyperlink ref="A226" r:id="rId198" tooltip="Topeka, Kansas" display="https://en.wikipedia.org/wiki/Topeka,_Kansas" xr:uid="{67481949-F882-464A-B6A6-626D32A82D50}"/>
+    <hyperlink ref="A227" r:id="rId199" tooltip="Wilmington, North Carolina" display="https://en.wikipedia.org/wiki/Wilmington,_North_Carolina" xr:uid="{2119452B-13EF-4892-9F66-943906FC84DF}"/>
+    <hyperlink ref="A228" r:id="rId200" tooltip="Lakeland, Florida" display="https://en.wikipedia.org/wiki/Lakeland,_Florida" xr:uid="{A1D87FDC-D554-48AC-995A-F6860FBD033E}"/>
+    <hyperlink ref="A229" r:id="rId201" tooltip="Thousand Oaks, California" display="https://en.wikipedia.org/wiki/Thousand_Oaks,_California" xr:uid="{603BAD32-8E4C-4D79-9C8D-5D0954FF0E9F}"/>
+    <hyperlink ref="A230" r:id="rId202" tooltip="Concord, California" display="https://en.wikipedia.org/wiki/Concord,_California" xr:uid="{ED78F782-2868-4B6D-BEDF-A272685AE35D}"/>
+    <hyperlink ref="A231" r:id="rId203" tooltip="Vallejo, California" display="https://en.wikipedia.org/wiki/Vallejo,_California" xr:uid="{7097017F-CF66-4243-B160-CF19DE3A2267}"/>
+    <hyperlink ref="A232" r:id="rId204" tooltip="Ann Arbor, Michigan" display="https://en.wikipedia.org/wiki/Ann_Arbor,_Michigan" xr:uid="{553E315B-35D3-44A6-A013-F1E8A0373A52}"/>
+    <hyperlink ref="A233" r:id="rId205" tooltip="Broken Arrow, Oklahoma" display="https://en.wikipedia.org/wiki/Broken_Arrow,_Oklahoma" xr:uid="{0059EE80-8A45-4D03-923A-B99BB1DF140D}"/>
+    <hyperlink ref="A234" r:id="rId206" tooltip="Fairfield, California" display="https://en.wikipedia.org/wiki/Fairfield,_California" xr:uid="{AFA3C10B-D1BB-4925-AA49-774FA576A43D}"/>
+    <hyperlink ref="A236" r:id="rId207" tooltip="Hartford, Connecticut" display="https://en.wikipedia.org/wiki/Hartford,_Connecticut" xr:uid="{1CF83A0B-54E4-4DFB-8F78-8220F113FE27}"/>
+    <hyperlink ref="A237" r:id="rId208" tooltip="Arvada, Colorado" display="https://en.wikipedia.org/wiki/Arvada,_Colorado" xr:uid="{E34E7BC9-DB14-4DC6-A62B-652BB8DC4F39}"/>
+    <hyperlink ref="A238" r:id="rId209" tooltip="Berkeley, California" display="https://en.wikipedia.org/wiki/Berkeley,_California" xr:uid="{F58A1B3A-1363-4070-A1DB-53CD2D8EA801}"/>
+    <hyperlink ref="A239" r:id="rId210" tooltip="Independence, Missouri" display="https://en.wikipedia.org/wiki/Independence,_Missouri" xr:uid="{9552DC8D-5E58-445D-8F54-557CAF5DC4F3}"/>
+    <hyperlink ref="A240" r:id="rId211" tooltip="Billings, Montana" display="https://en.wikipedia.org/wiki/Billings,_Montana" xr:uid="{CAC8EE67-B509-4FDF-B7F0-3C9C0015A709}"/>
+    <hyperlink ref="A241" r:id="rId212" tooltip="Cambridge, Massachusetts" display="https://en.wikipedia.org/wiki/Cambridge,_Massachusetts" xr:uid="{B6C026EF-7901-4ADD-AB65-B069FF3C8C5E}"/>
+    <hyperlink ref="A242" r:id="rId213" tooltip="Lowell, Massachusetts" display="https://en.wikipedia.org/wiki/Lowell,_Massachusetts" xr:uid="{1F945F81-C55B-4F0B-99E8-FBBB177CA02C}"/>
+    <hyperlink ref="A243" r:id="rId214" tooltip="Odessa, Texas" display="https://en.wikipedia.org/wiki/Odessa,_Texas" xr:uid="{610148C5-9861-4345-B74E-AE41B197C3D8}"/>
+    <hyperlink ref="A244" r:id="rId215" tooltip="High Point, North Carolina" display="https://en.wikipedia.org/wiki/High_Point,_North_Carolina" xr:uid="{9FB4C72E-5A47-4100-9E76-E5169ED9B159}"/>
+    <hyperlink ref="A245" r:id="rId216" tooltip="League City, Texas" display="https://en.wikipedia.org/wiki/League_City,_Texas" xr:uid="{F76F3E51-A8E8-47A8-99FF-B2D7E35759E6}"/>
+    <hyperlink ref="A246" r:id="rId217" tooltip="Antioch, California" display="https://en.wikipedia.org/wiki/Antioch,_California" xr:uid="{7C81C2F2-1150-4203-A0CD-960290CFDA84}"/>
+    <hyperlink ref="A247" r:id="rId218" tooltip="Richardson, Texas" display="https://en.wikipedia.org/wiki/Richardson,_Texas" xr:uid="{1EE11818-B344-464A-9CB9-57D1F85D5005}"/>
+    <hyperlink ref="A248" r:id="rId219" tooltip="Goodyear, Arizona" display="https://en.wikipedia.org/wiki/Goodyear,_Arizona" xr:uid="{BAEBEBD8-4ABB-4DD9-8DEB-998A37836DD0}"/>
+    <hyperlink ref="A249" r:id="rId220" tooltip="Pompano Beach, Florida" display="https://en.wikipedia.org/wiki/Pompano_Beach,_Florida" xr:uid="{CD0F4287-8AEE-4919-933A-DA0A384BB6E7}"/>
+    <hyperlink ref="A250" r:id="rId221" tooltip="Nampa, Idaho" display="https://en.wikipedia.org/wiki/Nampa,_Idaho" xr:uid="{550158AD-5E3F-41BB-A100-323D10DF3F8C}"/>
+    <hyperlink ref="A251" r:id="rId222" tooltip="Menifee, California" display="https://en.wikipedia.org/wiki/Menifee,_California" xr:uid="{296E559B-CC29-499E-BEE5-B4BAA9FE48CA}"/>
+    <hyperlink ref="A252" r:id="rId223" tooltip="Las Cruces, New Mexico" display="https://en.wikipedia.org/wiki/Las_Cruces,_New_Mexico" xr:uid="{E71D585B-BAB4-435C-994F-91A64FA21551}"/>
+    <hyperlink ref="A253" r:id="rId224" tooltip="Clearwater, Florida" display="https://en.wikipedia.org/wiki/Clearwater,_Florida" xr:uid="{B958717E-7CA8-43EC-B2B1-7B84B67DB9CF}"/>
+    <hyperlink ref="A254" r:id="rId225" tooltip="West Jordan, Utah" display="https://en.wikipedia.org/wiki/West_Jordan,_Utah" xr:uid="{F31A29F5-E17C-4EED-A6DA-85EA51C6270F}"/>
+    <hyperlink ref="A255" r:id="rId226" tooltip="New Braunfels, Texas" display="https://en.wikipedia.org/wiki/New_Braunfels,_Texas" xr:uid="{36227FAE-FC19-497F-A359-B256B6602824}"/>
+    <hyperlink ref="A256" r:id="rId227" tooltip="Manchester, New Hampshire" display="https://en.wikipedia.org/wiki/Manchester,_New_Hampshire" xr:uid="{18E7ED5D-3617-4BB3-990E-DC38DBBA9C71}"/>
+    <hyperlink ref="A257" r:id="rId228" tooltip="Miami Gardens, Florida" display="https://en.wikipedia.org/wiki/Miami_Gardens,_Florida" xr:uid="{04D4CFA2-AF3B-42F3-95F6-8CD0675767C5}"/>
+    <hyperlink ref="A258" r:id="rId229" tooltip="Waterbury, Connecticut" display="https://en.wikipedia.org/wiki/Waterbury,_Connecticut" xr:uid="{84C7295B-817B-472B-A4C0-C49A297B9A9A}"/>
+    <hyperlink ref="A259" r:id="rId230" tooltip="Provo, Utah" display="https://en.wikipedia.org/wiki/Provo,_Utah" xr:uid="{5AD91705-1191-4C84-AC0B-01D5EC8AC7F2}"/>
+    <hyperlink ref="A260" r:id="rId231" tooltip="Evansville, Indiana" display="https://en.wikipedia.org/wiki/Evansville,_Indiana" xr:uid="{3D93E37A-4A9F-4771-BD72-DDEB60DE23B9}"/>
+    <hyperlink ref="A261" r:id="rId232" tooltip="Westminster, Colorado" display="https://en.wikipedia.org/wiki/Westminster,_Colorado" xr:uid="{84D5954E-F995-42A0-B3A3-9181430599C4}"/>
+    <hyperlink ref="A262" r:id="rId233" tooltip="Elgin, Illinois" display="https://en.wikipedia.org/wiki/Elgin,_Illinois" xr:uid="{14C7D917-1DBD-4DBE-AB53-22E21388622F}"/>
+    <hyperlink ref="A263" r:id="rId234" tooltip="Conroe, Texas" display="https://en.wikipedia.org/wiki/Conroe,_Texas" xr:uid="{DD9C3E1A-980B-4666-9F2E-1D4952CCB128}"/>
+    <hyperlink ref="A264" r:id="rId235" tooltip="Greeley, Colorado" display="https://en.wikipedia.org/wiki/Greeley,_Colorado" xr:uid="{8CA4985B-2372-4D79-ACD7-4A4DE06DED0A}"/>
+    <hyperlink ref="A265" r:id="rId236" tooltip="Lansing, Michigan" display="https://en.wikipedia.org/wiki/Lansing,_Michigan" xr:uid="{2116C234-776D-4DB9-B3EB-83DD6B8F3FE3}"/>
+    <hyperlink ref="A266" r:id="rId237" tooltip="Buckeye, Arizona" display="https://en.wikipedia.org/wiki/Buckeye,_Arizona" xr:uid="{E0F4F41E-7A15-4A60-8E2D-5897BF290AFB}"/>
+    <hyperlink ref="A267" r:id="rId238" tooltip="Tuscaloosa, Alabama" display="https://en.wikipedia.org/wiki/Tuscaloosa,_Alabama" xr:uid="{D2EB49D3-2B35-47D9-A542-97AF06897478}"/>
+    <hyperlink ref="A268" r:id="rId239" tooltip="Allen, Texas" display="https://en.wikipedia.org/wiki/Allen,_Texas" xr:uid="{2043AED9-EE1B-4494-A41D-8667FB36610C}"/>
+    <hyperlink ref="A269" r:id="rId240" tooltip="Carlsbad, California" display="https://en.wikipedia.org/wiki/Carlsbad,_California" xr:uid="{23371DB8-7A80-4499-A75C-6DCDDC79CFEC}"/>
+    <hyperlink ref="A270" r:id="rId241" tooltip="Everett, Washington" display="https://en.wikipedia.org/wiki/Everett,_Washington" xr:uid="{128C008B-C6F6-46D6-B970-36D965AB5D36}"/>
+    <hyperlink ref="A271" r:id="rId242" tooltip="Beaumont, Texas" display="https://en.wikipedia.org/wiki/Beaumont,_Texas" xr:uid="{853FD3C3-E301-42C8-AF72-298737C51441}"/>
+    <hyperlink ref="A272" r:id="rId243" tooltip="Murrieta, California" display="https://en.wikipedia.org/wiki/Murrieta,_California" xr:uid="{8560D580-1E8B-4E59-9D71-FCFAD494DB60}"/>
+    <hyperlink ref="A273" r:id="rId244" tooltip="Rio Rancho, New Mexico" display="https://en.wikipedia.org/wiki/Rio_Rancho,_New_Mexico" xr:uid="{A1EF8FBB-23F3-4470-BFF8-0C16173BC62A}"/>
+    <hyperlink ref="A274" r:id="rId245" tooltip="Temecula, California" display="https://en.wikipedia.org/wiki/Temecula,_California" xr:uid="{F8C1865E-A75B-4898-A977-1D24561A1D8E}"/>
+    <hyperlink ref="A275" r:id="rId246" tooltip="Tyler, Texas" display="https://en.wikipedia.org/wiki/Tyler,_Texas" xr:uid="{7F383203-7C39-4212-978E-5A8AE462EDBC}"/>
+    <hyperlink ref="A276" r:id="rId247" tooltip="Davie, Florida" display="https://en.wikipedia.org/wiki/Davie,_Florida" xr:uid="{20723A51-8C85-444B-A75B-6638141CE779}"/>
+    <hyperlink ref="A277" r:id="rId248" tooltip="South Fulton, Georgia" display="https://en.wikipedia.org/wiki/South_Fulton,_Georgia" xr:uid="{73C75744-21C3-4146-B697-8210E551B66C}"/>
+    <hyperlink ref="A278" r:id="rId249" tooltip="Sparks, Nevada" display="https://en.wikipedia.org/wiki/Sparks,_Nevada" xr:uid="{6A4552ED-252D-4AB0-9EBE-8CC2E3115E5A}"/>
+    <hyperlink ref="A279" r:id="rId250" tooltip="Gresham, Oregon" display="https://en.wikipedia.org/wiki/Gresham,_Oregon" xr:uid="{ECC64D24-C00A-4C6B-B978-C093D8324F20}"/>
+    <hyperlink ref="A280" r:id="rId251" tooltip="Santa Maria, California" display="https://en.wikipedia.org/wiki/Santa_Maria,_California" xr:uid="{A888E5F6-EA84-4F58-A3B5-B0D41858EDFB}"/>
+    <hyperlink ref="A281" r:id="rId252" tooltip="Pueblo, Colorado" display="https://en.wikipedia.org/wiki/Pueblo,_Colorado" xr:uid="{2998C889-8570-45C1-9623-16B2D5FC4D32}"/>
+    <hyperlink ref="A282" r:id="rId253" tooltip="Hillsboro, Oregon" display="https://en.wikipedia.org/wiki/Hillsboro,_Oregon" xr:uid="{8327BC54-94CC-49B0-8051-C52DAB9F7A86}"/>
+    <hyperlink ref="A284" r:id="rId254" tooltip="Sugar Land, Texas" display="https://en.wikipedia.org/wiki/Sugar_Land,_Texas" xr:uid="{29F7F70C-FA86-4466-967B-A243148BA870}"/>
+    <hyperlink ref="A286" r:id="rId255" tooltip="Downey, California" display="https://en.wikipedia.org/wiki/Downey,_California" xr:uid="{B743D911-1E08-4AAC-8A82-105F6B0F1BD1}"/>
+    <hyperlink ref="A287" r:id="rId256" tooltip="Costa Mesa, California" display="https://en.wikipedia.org/wiki/Costa_Mesa,_California" xr:uid="{7A6973C9-C4E6-473B-BC32-E19FE8FF438C}"/>
+    <hyperlink ref="A288" r:id="rId257" tooltip="Centennial, Colorado" display="https://en.wikipedia.org/wiki/Centennial,_Colorado" xr:uid="{6327416D-84D1-47C4-B190-BF3E2A59BA2D}"/>
+    <hyperlink ref="A289" r:id="rId258" tooltip="Edinburg, Texas" display="https://en.wikipedia.org/wiki/Edinburg,_Texas" xr:uid="{2C9AFD68-19D2-4C61-8A4C-A20B6045ABB7}"/>
+    <hyperlink ref="A290" r:id="rId259" tooltip="Spokane Valley, Washington" display="https://en.wikipedia.org/wiki/Spokane_Valley,_Washington" xr:uid="{020B1BBE-B3DE-435B-83FD-DF7CED5056E8}"/>
+    <hyperlink ref="A291" r:id="rId260" tooltip="Jurupa Valley, California" display="https://en.wikipedia.org/wiki/Jurupa_Valley,_California" xr:uid="{295EA295-3E75-4397-AAFC-A719EF4437E8}"/>
+    <hyperlink ref="A292" r:id="rId261" tooltip="Bend, Oregon" display="https://en.wikipedia.org/wiki/Bend,_Oregon" xr:uid="{7E1F6E81-20AC-4E82-ADB7-017D2574DFD3}"/>
+    <hyperlink ref="A293" r:id="rId262" tooltip="West Covina, California" display="https://en.wikipedia.org/wiki/West_Covina,_California" xr:uid="{69575739-061B-4DA9-8FFC-159E9B3DA164}"/>
+    <hyperlink ref="A294" r:id="rId263" tooltip="Boulder, Colorado" display="https://en.wikipedia.org/wiki/Boulder,_Colorado" xr:uid="{48EB3296-B8FB-46E8-8D40-D1E2B21391D6}"/>
+    <hyperlink ref="A295" r:id="rId264" tooltip="Palm Coast, Florida" display="https://en.wikipedia.org/wiki/Palm_Coast,_Florida" xr:uid="{0DEF77AF-5FEB-4BB3-9800-CF76C6CB3653}"/>
+    <hyperlink ref="A296" r:id="rId265" tooltip="Lee's Summit, Missouri" display="https://en.wikipedia.org/wiki/Lee%27s_Summit,_Missouri" xr:uid="{CD41760B-D163-41AE-8194-32ED07FC2AB3}"/>
+    <hyperlink ref="A297" r:id="rId266" tooltip="Dearborn, Michigan" display="https://en.wikipedia.org/wiki/Dearborn,_Michigan" xr:uid="{E84116F0-6AE8-42B0-9503-2BF0ACE98582}"/>
+    <hyperlink ref="A298" r:id="rId267" tooltip="Green Bay, Wisconsin" display="https://en.wikipedia.org/wiki/Green_Bay,_Wisconsin" xr:uid="{BC32108E-8CCC-4531-A1AB-E0EFF02FC0DB}"/>
+    <hyperlink ref="A299" r:id="rId268" tooltip="St. George, Utah" display="https://en.wikipedia.org/wiki/St._George,_Utah" xr:uid="{0EF65130-5D66-4725-9CD9-9D5AEE02C313}"/>
+    <hyperlink ref="A301" r:id="rId269" tooltip="Brockton, Massachusetts" display="https://en.wikipedia.org/wiki/Brockton,_Massachusetts" xr:uid="{EE39A630-758B-4FAB-807D-AFF78DE08337}"/>
+    <hyperlink ref="A302" r:id="rId270" tooltip="Renton, Washington" display="https://en.wikipedia.org/wiki/Renton,_Washington" xr:uid="{00691DBE-1C7A-4929-8D13-7B896257CB2A}"/>
+    <hyperlink ref="A303" r:id="rId271" tooltip="Sandy Springs, Georgia" display="https://en.wikipedia.org/wiki/Sandy_Springs,_Georgia" xr:uid="{4EFA647B-2F55-44E4-8209-FC1F4AF9324B}"/>
+    <hyperlink ref="A304" r:id="rId272" tooltip="Rialto, California" display="https://en.wikipedia.org/wiki/Rialto,_California" xr:uid="{E501ED92-6B0C-4BE9-A742-5DE3A6B31C8F}"/>
+    <hyperlink ref="A305" r:id="rId273" tooltip="El Monte, California" display="https://en.wikipedia.org/wiki/El_Monte,_California" xr:uid="{ECB59E81-4A97-453D-8324-F9A4E42A8654}"/>
+    <hyperlink ref="A306" r:id="rId274" tooltip="Vacaville, California" display="https://en.wikipedia.org/wiki/Vacaville,_California" xr:uid="{44279042-4D9B-4080-AE32-A98C4C48B7A8}"/>
+    <hyperlink ref="A307" r:id="rId275" tooltip="Fishers, Indiana" display="https://en.wikipedia.org/wiki/Fishers,_Indiana" xr:uid="{402E2B4B-044E-41DF-915D-AB38ECD8AD70}"/>
+    <hyperlink ref="A308" r:id="rId276" tooltip="South Bend, Indiana" display="https://en.wikipedia.org/wiki/South_Bend,_Indiana" xr:uid="{73A00911-2D47-4E8A-A351-B4772D595DFE}"/>
+    <hyperlink ref="A309" r:id="rId277" tooltip="Carmel, Indiana" display="https://en.wikipedia.org/wiki/Carmel,_Indiana" xr:uid="{09A6F8BE-B0DF-4B38-820B-4B8794A44A5A}"/>
+    <hyperlink ref="A310" r:id="rId278" tooltip="Yuma, Arizona" display="https://en.wikipedia.org/wiki/Yuma,_Arizona" xr:uid="{39FF4BB3-6EEB-456E-BE88-EA97A18376E7}"/>
+    <hyperlink ref="A311" r:id="rId279" tooltip="Burbank, California" display="https://en.wikipedia.org/wiki/Burbank,_California" xr:uid="{6804245F-5620-40F0-8E47-04417D9DA751}"/>
+    <hyperlink ref="A312" r:id="rId280" tooltip="Lynn, Massachusetts" display="https://en.wikipedia.org/wiki/Lynn,_Massachusetts" xr:uid="{0737B5F0-2E3B-4CBF-9406-0EE9A67EF2B5}"/>
+    <hyperlink ref="A313" r:id="rId281" tooltip="Quincy, Massachusetts" display="https://en.wikipedia.org/wiki/Quincy,_Massachusetts" xr:uid="{8B0AAB2B-AA5C-4E2C-BA62-B9C8BAAF5207}"/>
+    <hyperlink ref="A314" r:id="rId282" tooltip="El Cajon, California" display="https://en.wikipedia.org/wiki/El_Cajon,_California" xr:uid="{9EDD555C-B7F6-40C9-B7E2-3B50F65F4560}"/>
+    <hyperlink ref="A316" r:id="rId283" tooltip="San Mateo, California" display="https://en.wikipedia.org/wiki/San_Mateo,_California" xr:uid="{A4DEEBC7-483A-48D5-9277-289D8F450BDB}"/>
+    <hyperlink ref="A317" r:id="rId284" tooltip="Chico, California" display="https://en.wikipedia.org/wiki/Chico,_California" xr:uid="{CD6EB241-A61E-4451-A74A-CA5412254C62}"/>
+    <hyperlink ref="A318" r:id="rId285" tooltip="Inglewood, California" display="https://en.wikipedia.org/wiki/Inglewood,_California" xr:uid="{88256F8E-1302-4138-BFEA-37C5A32B5E51}"/>
+    <hyperlink ref="A319" r:id="rId286" tooltip="Wichita Falls, Texas" display="https://en.wikipedia.org/wiki/Wichita_Falls,_Texas" xr:uid="{6F93A719-EED6-4A9C-B438-4DE9D8E12E70}"/>
+    <hyperlink ref="A320" r:id="rId287" tooltip="Boca Raton, Florida" display="https://en.wikipedia.org/wiki/Boca_Raton,_Florida" xr:uid="{40086BB0-4537-4537-8A7F-AD1DB13E49F1}"/>
+    <hyperlink ref="A321" r:id="rId288" tooltip="Hesperia, California" display="https://en.wikipedia.org/wiki/Hesperia,_California" xr:uid="{5A282B4D-DB62-4EDE-9251-B12B80A02CF6}"/>
+    <hyperlink ref="A322" r:id="rId289" tooltip="Daly City, California" display="https://en.wikipedia.org/wiki/Daly_City,_California" xr:uid="{273F395E-8A2C-4A59-B9C0-6BBAF95CE82C}"/>
+    <hyperlink ref="A324" r:id="rId290" tooltip="Georgetown, Texas" display="https://en.wikipedia.org/wiki/Georgetown,_Texas" xr:uid="{F6B17462-7C74-498E-B740-65A4E7749CE7}"/>
+    <hyperlink ref="A325" r:id="rId291" tooltip="New Bedford, Massachusetts" display="https://en.wikipedia.org/wiki/New_Bedford,_Massachusetts" xr:uid="{25990844-1D54-45CB-A483-30DD8FBB0CD2}"/>
+    <hyperlink ref="A326" r:id="rId292" tooltip="Albany, New York" display="https://en.wikipedia.org/wiki/Albany,_New_York" xr:uid="{134E9866-C107-4A21-AECB-C63388B25232}"/>
+    <hyperlink ref="A327" r:id="rId293" tooltip="Davenport, Iowa" display="https://en.wikipedia.org/wiki/Davenport,_Iowa" xr:uid="{ABF3CE13-C477-4AD0-92A4-19A33CE8505D}"/>
+    <hyperlink ref="A328" r:id="rId294" tooltip="Plantation, Florida" display="https://en.wikipedia.org/wiki/Plantation,_Florida" xr:uid="{F9A40EA9-2F97-41AC-9CB0-6C87E2448DA0}"/>
+    <hyperlink ref="A329" r:id="rId295" tooltip="Deltona, Florida" display="https://en.wikipedia.org/wiki/Deltona,_Florida" xr:uid="{F86B9F1E-0353-40B1-87DA-D74935E2F1E2}"/>
+    <hyperlink ref="A330" r:id="rId296" tooltip="Federal Way, Washington" display="https://en.wikipedia.org/wiki/Federal_Way,_Washington" xr:uid="{6A733CDF-C6F6-4A3F-86ED-0B1C45801AEA}"/>
+    <hyperlink ref="A331" r:id="rId297" tooltip="San Angelo, Texas" display="https://en.wikipedia.org/wiki/San_Angelo,_Texas" xr:uid="{BF3DB560-73FF-4047-A1A3-D9F70CDFC2F0}"/>
+    <hyperlink ref="A332" r:id="rId298" tooltip="Tracy, California" display="https://en.wikipedia.org/wiki/Tracy,_California" xr:uid="{690292EE-71CB-4C84-8011-880C6516847C}"/>
+    <hyperlink ref="A333" r:id="rId299" tooltip="Sunrise, Florida" display="https://en.wikipedia.org/wiki/Sunrise,_Florida" xr:uid="{D6743DD7-E0E4-4D89-9538-92361E1ED4C2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId311"/>
+  <drawing r:id="rId300"/>
 </worksheet>
 </file>
</xml_diff>